<commit_message>
Complete exact-handoff reset recovery and successor connected controls
</commit_message>
<xml_diff>
--- a/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
+++ b/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
@@ -546,25 +546,25 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="14">
-    <x:tableColumn id="1" name="Case ID"/>
-    <x:tableColumn id="2" name="Control ID"/>
-    <x:tableColumn id="3" name="Jurisdiction"/>
-    <x:tableColumn id="4" name="Entity / exact route"/>
-    <x:tableColumn id="5" name="Local / component / outcome variant"/>
-    <x:tableColumn id="6" name="Channel"/>
-    <x:tableColumn id="7" name="Locale"/>
-    <x:tableColumn id="8" name="Candidate / config version"/>
-    <x:tableColumn id="9" name="Status"/>
-    <x:tableColumn id="10" name="Observed result"/>
-    <x:tableColumn id="11" name="Evidence locator"/>
-    <x:tableColumn id="12" name="Reviewer"/>
-    <x:tableColumn id="13" name="Defect ID"/>
-    <x:tableColumn id="14" name="N/A or reuse rationale"/>
-  </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</x:table>
+<ns0:table xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <ns0:tableColumns count="14">
+    <ns0:tableColumn id="1" name="Case ID"/>
+    <ns0:tableColumn id="2" name="Control ID"/>
+    <ns0:tableColumn id="3" name="Jurisdiction"/>
+    <ns0:tableColumn id="4" name="Entity / exact route"/>
+    <ns0:tableColumn id="5" name="Local / component / outcome variant"/>
+    <ns0:tableColumn id="6" name="Channel"/>
+    <ns0:tableColumn id="7" name="Locale"/>
+    <ns0:tableColumn id="8" name="Candidate / config version"/>
+    <ns0:tableColumn id="9" name="Status"/>
+    <ns0:tableColumn id="10" name="Observed result"/>
+    <ns0:tableColumn id="11" name="Evidence locator"/>
+    <ns0:tableColumn id="12" name="Reviewer"/>
+    <ns0:tableColumn id="13" name="Defect ID"/>
+    <ns0:tableColumn id="14" name="N/A or reuse rationale"/>
+  </ns0:tableColumns>
+  <ns0:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</ns0:table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
@@ -608,22 +608,22 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="QADefects" displayName="QADefects" ref="A4:K5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="11">
-    <x:tableColumn id="1" name="Defect ID"/>
-    <x:tableColumn id="2" name="Severity"/>
-    <x:tableColumn id="3" name="Affected case IDs"/>
-    <x:tableColumn id="4" name="Expected vs actual"/>
-    <x:tableColumn id="5" name="Reproduction / evidence"/>
-    <x:tableColumn id="6" name="Existing issue / owner"/>
-    <x:tableColumn id="7" name="State"/>
-    <x:tableColumn id="8" name="Fix candidate"/>
-    <x:tableColumn id="9" name="Retest evidence"/>
-    <x:tableColumn id="10" name="Shared blast radius"/>
-    <x:tableColumn id="11" name="Scope / decision notes"/>
-  </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</x:table>
+<ns0:table xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="QADefects" displayName="QADefects" ref="A4:K9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <ns0:tableColumns count="11">
+    <ns0:tableColumn id="1" name="Defect ID"/>
+    <ns0:tableColumn id="2" name="Severity"/>
+    <ns0:tableColumn id="3" name="Affected case IDs"/>
+    <ns0:tableColumn id="4" name="Expected vs actual"/>
+    <ns0:tableColumn id="5" name="Reproduction / evidence"/>
+    <ns0:tableColumn id="6" name="Existing issue / owner"/>
+    <ns0:tableColumn id="7" name="State"/>
+    <ns0:tableColumn id="8" name="Fix candidate"/>
+    <ns0:tableColumn id="9" name="Retest evidence"/>
+    <ns0:tableColumn id="10" name="Shared blast radius"/>
+    <ns0:tableColumn id="11" name="Scope / decision notes"/>
+  </ns0:tableColumns>
+  <ns0:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</ns0:table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
@@ -8397,159 +8397,431 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="40" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="40" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="34" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="20" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="40" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="40" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="20" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="16" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="40" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="32" customHeight="1">
-      <x:c r="A1" s="3" t="str">
-        <x:v>FINAL QA / EXECUTION INSTANCES</x:v>
-      </x:c>
-      <x:c r="B1" s="3"/>
-      <x:c r="C1" s="3"/>
-      <x:c r="D1" s="3"/>
-      <x:c r="E1" s="3"/>
-      <x:c r="F1" s="3"/>
-      <x:c r="G1" s="3"/>
-      <x:c r="H1" s="3"/>
-      <x:c r="I1" s="3"/>
-      <x:c r="J1" s="3"/>
-      <x:c r="K1" s="3"/>
-      <x:c r="L1" s="3"/>
-      <x:c r="M1" s="3"/>
-      <x:c r="N1" s="3"/>
-    </x:row>
-    <x:row r="2" ht="44" customHeight="1">
-      <x:c r="A2" s="7" t="str">
-        <x:v>Populate at P00 from actual scope. One row per Control × Entity × meaningful Variant. Add rows to this table (no fixed count limit). Missing/blocked/stale/skipped is never PASS.</x:v>
-      </x:c>
-      <x:c r="B2" s="7"/>
-      <x:c r="C2" s="7"/>
-      <x:c r="D2" s="7"/>
-      <x:c r="E2" s="7"/>
-      <x:c r="F2" s="7"/>
-      <x:c r="G2" s="7"/>
-      <x:c r="H2" s="7"/>
-      <x:c r="I2" s="7"/>
-      <x:c r="J2" s="7"/>
-      <x:c r="K2" s="7"/>
-      <x:c r="L2" s="7"/>
-      <x:c r="M2" s="7"/>
-      <x:c r="N2" s="7"/>
-    </x:row>
-    <x:row r="4" ht="32" customHeight="1">
-      <x:c r="A4" s="18" t="str">
-        <x:v>Case ID</x:v>
-      </x:c>
-      <x:c r="B4" s="18" t="str">
-        <x:v>Control ID</x:v>
-      </x:c>
-      <x:c r="C4" s="18" t="str">
-        <x:v>Jurisdiction</x:v>
-      </x:c>
-      <x:c r="D4" s="18" t="str">
-        <x:v>Entity / exact route</x:v>
-      </x:c>
-      <x:c r="E4" s="18" t="str">
-        <x:v>Local / component / outcome variant</x:v>
-      </x:c>
-      <x:c r="F4" s="18" t="str">
-        <x:v>Channel</x:v>
-      </x:c>
-      <x:c r="G4" s="18" t="str">
-        <x:v>Locale</x:v>
-      </x:c>
-      <x:c r="H4" s="18" t="str">
-        <x:v>Candidate / config version</x:v>
-      </x:c>
-      <x:c r="I4" s="18" t="str">
-        <x:v>Status</x:v>
-      </x:c>
-      <x:c r="J4" s="18" t="str">
-        <x:v>Observed result</x:v>
-      </x:c>
-      <x:c r="K4" s="18" t="str">
-        <x:v>Evidence locator</x:v>
-      </x:c>
-      <x:c r="L4" s="18" t="str">
-        <x:v>Reviewer</x:v>
-      </x:c>
-      <x:c r="M4" s="18" t="str">
-        <x:v>Defect ID</x:v>
-      </x:c>
-      <x:c r="N4" s="18" t="str">
-        <x:v>N/A or reuse rationale</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="82" customHeight="1">
-      <x:c r="A5" s="12"/>
-      <x:c r="B5" s="12"/>
-      <x:c r="C5" s="12"/>
-      <x:c r="D5" s="12"/>
-      <x:c r="E5" s="12"/>
-      <x:c r="F5" s="12"/>
-      <x:c r="G5" s="12"/>
-      <x:c r="H5" s="12"/>
-      <x:c r="I5" s="12"/>
-      <x:c r="J5" s="12"/>
-      <x:c r="K5" s="12"/>
-      <x:c r="L5" s="12"/>
-      <x:c r="M5" s="12"/>
-      <x:c r="N5" s="12"/>
-    </x:row>
-  </x:sheetData>
-  <x:mergeCells>
-    <x:mergeCell ref="A1:N1"/>
-    <x:mergeCell ref="A2:N2"/>
-  </x:mergeCells>
-  <x:conditionalFormatting sqref="I5:I1000">
-    <x:cfRule type="expression" dxfId="10" priority="1">
-      <x:formula>I5="PASS"</x:formula>
-    </x:cfRule>
-    <x:cfRule type="expression" dxfId="11" priority="2">
-      <x:formula>I5="FAIL"</x:formula>
-    </x:cfRule>
-    <x:cfRule type="expression" dxfId="12" priority="3">
-      <x:formula>I5="BLOCKED"</x:formula>
-    </x:cfRule>
-    <x:cfRule type="expression" dxfId="13" priority="4">
-      <x:formula>I5="STALE"</x:formula>
-    </x:cfRule>
-    <x:cfRule type="expression" dxfId="14" priority="5">
-      <x:formula>I5="IN PROGRESS"</x:formula>
-    </x:cfRule>
-  </x:conditionalFormatting>
-  <x:dataValidations count="3">
-    <x:dataValidation type="list" sqref="I5:I1000">
-      <x:formula1>"NOT RUN,IN PROGRESS,PASS,FAIL,BLOCKED,NOT APPLICABLE,STALE"</x:formula1>
-    </x:dataValidation>
-    <x:dataValidation type="list" sqref="F5:F1000">
-      <x:formula1>"DTC,RCAP,Standard Clinic,Legal Aid Clinic,Public,Internal,Shared"</x:formula1>
-    </x:dataValidation>
-    <x:dataValidation type="list" sqref="G5:G1000">
-      <x:formula1>"EN,ES,BOTH,N/A"</x:formula1>
-    </x:dataValidation>
-  </x:dataValidations>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f81d841fff147e3"/>
-  </x:tableParts>
-</x:worksheet>
+<ns0:worksheet xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <ns0:sheetFormatPr defaultRowHeight="15"/>
+  <ns0:cols>
+    <ns0:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <ns0:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
+    <ns0:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
+    <ns0:col min="4" max="4" width="40" hidden="0" customWidth="1"/>
+    <ns0:col min="5" max="5" width="40" hidden="0" customWidth="1"/>
+    <ns0:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <ns0:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
+    <ns0:col min="8" max="8" width="34" hidden="0" customWidth="1"/>
+    <ns0:col min="9" max="9" width="20" hidden="0" customWidth="1"/>
+    <ns0:col min="10" max="10" width="40" hidden="0" customWidth="1"/>
+    <ns0:col min="11" max="11" width="40" hidden="0" customWidth="1"/>
+    <ns0:col min="12" max="12" width="20" hidden="0" customWidth="1"/>
+    <ns0:col min="13" max="13" width="16" hidden="0" customWidth="1"/>
+    <ns0:col min="14" max="14" width="40" hidden="0" customWidth="1"/>
+  </ns0:cols>
+  <ns0:sheetData>
+    <ns0:row r="1" ht="32" customHeight="1">
+      <ns0:c r="A1" s="3" t="str">
+        <ns0:v>FINAL QA / EXECUTION INSTANCES</ns0:v>
+      </ns0:c>
+      <ns0:c r="B1" s="3"/>
+      <ns0:c r="C1" s="3"/>
+      <ns0:c r="D1" s="3"/>
+      <ns0:c r="E1" s="3"/>
+      <ns0:c r="F1" s="3"/>
+      <ns0:c r="G1" s="3"/>
+      <ns0:c r="H1" s="3"/>
+      <ns0:c r="I1" s="3"/>
+      <ns0:c r="J1" s="3"/>
+      <ns0:c r="K1" s="3"/>
+      <ns0:c r="L1" s="3"/>
+      <ns0:c r="M1" s="3"/>
+      <ns0:c r="N1" s="3"/>
+    </ns0:row>
+    <ns0:row r="2" ht="44" customHeight="1">
+      <ns0:c r="A2" s="7" t="str">
+        <ns0:v>Populate at P00 from actual scope. One row per Control × Entity × meaningful Variant. Add rows to this table (no fixed count limit). Missing/blocked/stale/skipped is never PASS.</ns0:v>
+      </ns0:c>
+      <ns0:c r="B2" s="7"/>
+      <ns0:c r="C2" s="7"/>
+      <ns0:c r="D2" s="7"/>
+      <ns0:c r="E2" s="7"/>
+      <ns0:c r="F2" s="7"/>
+      <ns0:c r="G2" s="7"/>
+      <ns0:c r="H2" s="7"/>
+      <ns0:c r="I2" s="7"/>
+      <ns0:c r="J2" s="7"/>
+      <ns0:c r="K2" s="7"/>
+      <ns0:c r="L2" s="7"/>
+      <ns0:c r="M2" s="7"/>
+      <ns0:c r="N2" s="7"/>
+    </ns0:row>
+    <ns0:row r="4" ht="32" customHeight="1">
+      <ns0:c r="A4" s="18" t="str">
+        <ns0:v>Case ID</ns0:v>
+      </ns0:c>
+      <ns0:c r="B4" s="18" t="str">
+        <ns0:v>Control ID</ns0:v>
+      </ns0:c>
+      <ns0:c r="C4" s="18" t="str">
+        <ns0:v>Jurisdiction</ns0:v>
+      </ns0:c>
+      <ns0:c r="D4" s="18" t="str">
+        <ns0:v>Entity / exact route</ns0:v>
+      </ns0:c>
+      <ns0:c r="E4" s="18" t="str">
+        <ns0:v>Local / component / outcome variant</ns0:v>
+      </ns0:c>
+      <ns0:c r="F4" s="18" t="str">
+        <ns0:v>Channel</ns0:v>
+      </ns0:c>
+      <ns0:c r="G4" s="18" t="str">
+        <ns0:v>Locale</ns0:v>
+      </ns0:c>
+      <ns0:c r="H4" s="18" t="str">
+        <ns0:v>Candidate / config version</ns0:v>
+      </ns0:c>
+      <ns0:c r="I4" s="18" t="str">
+        <ns0:v>Status</ns0:v>
+      </ns0:c>
+      <ns0:c r="J4" s="18" t="str">
+        <ns0:v>Observed result</ns0:v>
+      </ns0:c>
+      <ns0:c r="K4" s="18" t="str">
+        <ns0:v>Evidence locator</ns0:v>
+      </ns0:c>
+      <ns0:c r="L4" s="18" t="str">
+        <ns0:v>Reviewer</ns0:v>
+      </ns0:c>
+      <ns0:c r="M4" s="18" t="str">
+        <ns0:v>Defect ID</ns0:v>
+      </ns0:c>
+      <ns0:c r="N4" s="18" t="str">
+        <ns0:v>N/A or reuse rationale</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="5">
+      <ns0:c r="A5" t="inlineStr">
+        <ns0:is>
+          <ns0:t>D4-RECOVERY-F1F2</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B5" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P08-08</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C5" t="inlineStr">
+        <ns0:is>
+          <ns0:t>All 51</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D5" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Clinic reset prepare/close/complete</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E5" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Network/preparation/expiry/re-auth/reload faults</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F5" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Shared</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G5" t="inlineStr">
+        <ns0:is>
+          <ns0:t>EN</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H5" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Amendment commit containing this record</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I5" t="inlineStr">
+        <ns0:is>
+          <ns0:t>IN PROGRESS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J5" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Local controls pass; independent review and hosted scope pending</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K5" t="inlineStr">
+        <ns0:is>
+          <ns0:t>CODEX_D3_D4_PRODUCT_SUCCESSOR_REVISION/REVIEW.md</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L5" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Claude review pending</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M5" t="inlineStr">
+        <ns0:is>
+          <ns0:t>CLAUDE-4723-F1-F2</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N5" t="inlineStr">
+        <ns0:is>
+          <ns0:t>D3 implementation unchanged</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="6">
+      <ns0:c r="A6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>D4-ENTRY-F4</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P08-08</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>All 51</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>/clinic/reset; /clinic; /clinic/&lt;eventSlug&gt;</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Canonical event association; missing/invalid context</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Shared</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>EN</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Amendment commit containing this record</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>IN PROGRESS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Actual product routes in compiled/browser controls</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>CODEX_D3_D4_PRODUCT_SUCCESSOR_REVISION/REVIEW.md</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Claude review pending</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>CLAUDE-4723-F4</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>No synthetic success landing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="7">
+      <ns0:c r="A7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>D4-BOUNDARY-O3</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P09-17</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>All 51</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Proxy documents/RSC/private APIs</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Locked response, not DOM mask</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Shared</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>EN</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Amendment commit containing this record</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>IN PROGRESS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Full-build HTTP evidence in revision package</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>CODEX_D3_D4_PRODUCT_SUCCESSOR_REVISION/evidence/full-build-boundary.log</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Claude review pending</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>CLAUDE-4723-O3</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Marker restricts; does not authorize</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="8">
+      <ns0:c r="A8" t="inlineStr">
+        <ns0:is>
+          <ns0:t>D4-CONNECTED-F3</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B8" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P09-01</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C8" t="inlineStr">
+        <ns0:is>
+          <ns0:t>All 51</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D8" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Current endpoint lifecycle</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E8" t="inlineStr">
+        <ns0:is>
+          <ns0:t>D1 preventive denial; D2 shutdown; canonical PG closure</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F8" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Shared</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G8" t="inlineStr">
+        <ns0:is>
+          <ns0:t>EN</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H8" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Amendment commit containing this record</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I8" t="inlineStr">
+        <ns0:is>
+          <ns0:t>IN PROGRESS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J8" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Current connected positive/negative controls; historical fixture separately pinned</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K8" t="inlineStr">
+        <ns0:is>
+          <ns0:t>CODEX_D3_D4_PRODUCT_SUCCESSOR_REVISION/evidence/connected-successor.log</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L8" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Claude review pending</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M8" t="inlineStr">
+        <ns0:is>
+          <ns0:t>CLAUDE-4723-F3</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N8" t="inlineStr">
+        <ns0:is>
+          <ns0:t>No hosted checkpoint repin</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+  </ns0:sheetData>
+  <ns0:mergeCells>
+    <ns0:mergeCell ref="A1:N1"/>
+    <ns0:mergeCell ref="A2:N2"/>
+  </ns0:mergeCells>
+  <ns0:conditionalFormatting sqref="I5:I1000">
+    <ns0:cfRule type="expression" dxfId="10" priority="1">
+      <ns0:formula>I5="PASS"</ns0:formula>
+    </ns0:cfRule>
+    <ns0:cfRule type="expression" dxfId="11" priority="2">
+      <ns0:formula>I5="FAIL"</ns0:formula>
+    </ns0:cfRule>
+    <ns0:cfRule type="expression" dxfId="12" priority="3">
+      <ns0:formula>I5="BLOCKED"</ns0:formula>
+    </ns0:cfRule>
+    <ns0:cfRule type="expression" dxfId="13" priority="4">
+      <ns0:formula>I5="STALE"</ns0:formula>
+    </ns0:cfRule>
+    <ns0:cfRule type="expression" dxfId="14" priority="5">
+      <ns0:formula>I5="IN PROGRESS"</ns0:formula>
+    </ns0:cfRule>
+  </ns0:conditionalFormatting>
+  <ns0:dataValidations count="3">
+    <ns0:dataValidation type="list" sqref="I5:I1000">
+      <ns0:formula1>"NOT RUN,IN PROGRESS,PASS,FAIL,BLOCKED,NOT APPLICABLE,STALE"</ns0:formula1>
+    </ns0:dataValidation>
+    <ns0:dataValidation type="list" sqref="F5:F1000">
+      <ns0:formula1>"DTC,RCAP,Standard Clinic,Legal Aid Clinic,Public,Internal,Shared"</ns0:formula1>
+    </ns0:dataValidation>
+    <ns0:dataValidation type="list" sqref="G5:G1000">
+      <ns0:formula1>"EN,ES,BOTH,N/A"</ns0:formula1>
+    </ns0:dataValidation>
+  </ns0:dataValidations>
+  <ns0:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ns0:tableParts count="1">
+    <ns0:tablePart ns1:id="R9f81d841fff147e3"/>
+  </ns0:tableParts>
+</ns0:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
@@ -10544,118 +10816,390 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="40" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="40" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="32" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="22" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="32" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="40" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="40" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="40" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="32" customHeight="1">
-      <x:c r="A1" s="3" t="str">
-        <x:v>FINAL QA / DEFECTS AND RETEST</x:v>
-      </x:c>
-      <x:c r="B1" s="3"/>
-      <x:c r="C1" s="3"/>
-      <x:c r="D1" s="3"/>
-      <x:c r="E1" s="3"/>
-      <x:c r="F1" s="3"/>
-      <x:c r="G1" s="3"/>
-      <x:c r="H1" s="3"/>
-      <x:c r="I1" s="3"/>
-      <x:c r="J1" s="3"/>
-      <x:c r="K1" s="3"/>
-    </x:row>
-    <x:row r="2" ht="44" customHeight="1">
-      <x:c r="A2" s="7" t="str">
-        <x:v>Link to the existing build issue where available. Severity never waives a required check. One root may affect many cases; every affected instance remains visible until retested.</x:v>
-      </x:c>
-      <x:c r="B2" s="7"/>
-      <x:c r="C2" s="7"/>
-      <x:c r="D2" s="7"/>
-      <x:c r="E2" s="7"/>
-      <x:c r="F2" s="7"/>
-      <x:c r="G2" s="7"/>
-      <x:c r="H2" s="7"/>
-      <x:c r="I2" s="7"/>
-      <x:c r="J2" s="7"/>
-      <x:c r="K2" s="7"/>
-    </x:row>
-    <x:row r="4" ht="32" customHeight="1">
-      <x:c r="A4" s="18" t="str">
-        <x:v>Defect ID</x:v>
-      </x:c>
-      <x:c r="B4" s="18" t="str">
-        <x:v>Severity</x:v>
-      </x:c>
-      <x:c r="C4" s="18" t="str">
-        <x:v>Affected case IDs</x:v>
-      </x:c>
-      <x:c r="D4" s="18" t="str">
-        <x:v>Expected vs actual</x:v>
-      </x:c>
-      <x:c r="E4" s="18" t="str">
-        <x:v>Reproduction / evidence</x:v>
-      </x:c>
-      <x:c r="F4" s="18" t="str">
-        <x:v>Existing issue / owner</x:v>
-      </x:c>
-      <x:c r="G4" s="18" t="str">
-        <x:v>State</x:v>
-      </x:c>
-      <x:c r="H4" s="18" t="str">
-        <x:v>Fix candidate</x:v>
-      </x:c>
-      <x:c r="I4" s="18" t="str">
-        <x:v>Retest evidence</x:v>
-      </x:c>
-      <x:c r="J4" s="18" t="str">
-        <x:v>Shared blast radius</x:v>
-      </x:c>
-      <x:c r="K4" s="18" t="str">
-        <x:v>Scope / decision notes</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="94" customHeight="1">
-      <x:c r="A5" s="12"/>
-      <x:c r="B5" s="12"/>
-      <x:c r="C5" s="12"/>
-      <x:c r="D5" s="12"/>
-      <x:c r="E5" s="12"/>
-      <x:c r="F5" s="12"/>
-      <x:c r="G5" s="12"/>
-      <x:c r="H5" s="12"/>
-      <x:c r="I5" s="12"/>
-      <x:c r="J5" s="12"/>
-      <x:c r="K5" s="12"/>
-    </x:row>
-  </x:sheetData>
-  <x:mergeCells>
-    <x:mergeCell ref="A1:K1"/>
-    <x:mergeCell ref="A2:K2"/>
-  </x:mergeCells>
-  <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="B5:B1000">
-      <x:formula1>"S0,S1,S2,S3"</x:formula1>
-    </x:dataValidation>
-    <x:dataValidation type="list" sqref="G5:G1000">
-      <x:formula1>"OPEN,ASSIGNED,FIXED AWAITING RETEST,CLOSED,BLOCKED"</x:formula1>
-    </x:dataValidation>
-  </x:dataValidations>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R087daac7a3394538"/>
-  </x:tableParts>
-</x:worksheet>
+<ns0:worksheet xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <ns0:sheetFormatPr defaultRowHeight="15"/>
+  <ns0:cols>
+    <ns0:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <ns0:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
+    <ns0:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
+    <ns0:col min="4" max="4" width="40" hidden="0" customWidth="1"/>
+    <ns0:col min="5" max="5" width="40" hidden="0" customWidth="1"/>
+    <ns0:col min="6" max="6" width="32" hidden="0" customWidth="1"/>
+    <ns0:col min="7" max="7" width="22" hidden="0" customWidth="1"/>
+    <ns0:col min="8" max="8" width="32" hidden="0" customWidth="1"/>
+    <ns0:col min="9" max="9" width="40" hidden="0" customWidth="1"/>
+    <ns0:col min="10" max="10" width="40" hidden="0" customWidth="1"/>
+    <ns0:col min="11" max="11" width="40" hidden="0" customWidth="1"/>
+  </ns0:cols>
+  <ns0:sheetData>
+    <ns0:row r="1" ht="32" customHeight="1">
+      <ns0:c r="A1" s="3" t="str">
+        <ns0:v>FINAL QA / DEFECTS AND RETEST</ns0:v>
+      </ns0:c>
+      <ns0:c r="B1" s="3"/>
+      <ns0:c r="C1" s="3"/>
+      <ns0:c r="D1" s="3"/>
+      <ns0:c r="E1" s="3"/>
+      <ns0:c r="F1" s="3"/>
+      <ns0:c r="G1" s="3"/>
+      <ns0:c r="H1" s="3"/>
+      <ns0:c r="I1" s="3"/>
+      <ns0:c r="J1" s="3"/>
+      <ns0:c r="K1" s="3"/>
+    </ns0:row>
+    <ns0:row r="2" ht="44" customHeight="1">
+      <ns0:c r="A2" s="7" t="str">
+        <ns0:v>Link to the existing build issue where available. Severity never waives a required check. One root may affect many cases; every affected instance remains visible until retested.</ns0:v>
+      </ns0:c>
+      <ns0:c r="B2" s="7"/>
+      <ns0:c r="C2" s="7"/>
+      <ns0:c r="D2" s="7"/>
+      <ns0:c r="E2" s="7"/>
+      <ns0:c r="F2" s="7"/>
+      <ns0:c r="G2" s="7"/>
+      <ns0:c r="H2" s="7"/>
+      <ns0:c r="I2" s="7"/>
+      <ns0:c r="J2" s="7"/>
+      <ns0:c r="K2" s="7"/>
+    </ns0:row>
+    <ns0:row r="4" ht="32" customHeight="1">
+      <ns0:c r="A4" s="18" t="str">
+        <ns0:v>Defect ID</ns0:v>
+      </ns0:c>
+      <ns0:c r="B4" s="18" t="str">
+        <ns0:v>Severity</ns0:v>
+      </ns0:c>
+      <ns0:c r="C4" s="18" t="str">
+        <ns0:v>Affected case IDs</ns0:v>
+      </ns0:c>
+      <ns0:c r="D4" s="18" t="str">
+        <ns0:v>Expected vs actual</ns0:v>
+      </ns0:c>
+      <ns0:c r="E4" s="18" t="str">
+        <ns0:v>Reproduction / evidence</ns0:v>
+      </ns0:c>
+      <ns0:c r="F4" s="18" t="str">
+        <ns0:v>Existing issue / owner</ns0:v>
+      </ns0:c>
+      <ns0:c r="G4" s="18" t="str">
+        <ns0:v>State</ns0:v>
+      </ns0:c>
+      <ns0:c r="H4" s="18" t="str">
+        <ns0:v>Fix candidate</ns0:v>
+      </ns0:c>
+      <ns0:c r="I4" s="18" t="str">
+        <ns0:v>Retest evidence</ns0:v>
+      </ns0:c>
+      <ns0:c r="J4" s="18" t="str">
+        <ns0:v>Shared blast radius</ns0:v>
+      </ns0:c>
+      <ns0:c r="K4" s="18" t="str">
+        <ns0:v>Scope / decision notes</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="5">
+      <ns0:c r="A5" t="inlineStr">
+        <ns0:is>
+          <ns0:t>CLAUDE-4723-F1-F2</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B5" t="inlineStr">
+        <ns0:is>
+          <ns0:t>S1</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C5" t="inlineStr">
+        <ns0:is>
+          <ns0:t>D4-RECOVERY-F1F2</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D5" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Failed preparation and expiry must preserve authorized completion</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E5" t="inlineStr">
+        <ns0:is>
+          <ns0:t>CLAUDE_PRODUCT_REVIEW_4723f603 and readiness addendum</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F5" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Existing productSuccessor work item / Codex</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G5" t="inlineStr">
+        <ns0:is>
+          <ns0:t>FIXED AWAITING RETEST</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H5" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Amendment commit containing this record</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I5" t="inlineStr">
+        <ns0:is>
+          <ns0:t>CODEX_D3_D4_PRODUCT_SUCCESSOR_REVISION/REVIEW.md</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J5" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Shared Clinic / dependent controls</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K5" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Independent review and hosted acceptance not waived</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="6">
+      <ns0:c r="A6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>CLAUDE-4723-F3</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>S2</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>D4-CONNECTED-F3</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Successor connected proof must exercise current lifecycle</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>CLAUDE_PRODUCT_REVIEW_4723f603 and readiness addendum</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Existing productSuccessor work item / Codex</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>FIXED AWAITING RETEST</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Amendment commit containing this record</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>CODEX_D3_D4_PRODUCT_SUCCESSOR_REVISION/REVIEW.md</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Shared Clinic / dependent controls</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K6" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Independent review and hosted acceptance not waived</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="7">
+      <ns0:c r="A7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>CLAUDE-4723-F4</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>S2</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>D4-ENTRY-F4</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Reload recovery must retain original event and reach actual entry</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>CLAUDE_PRODUCT_REVIEW_4723f603 and readiness addendum</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Existing productSuccessor work item / Codex</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>FIXED AWAITING RETEST</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Amendment commit containing this record</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>CODEX_D3_D4_PRODUCT_SUCCESSOR_REVISION/REVIEW.md</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Shared Clinic / dependent controls</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K7" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Independent review and hosted acceptance not waived</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="8">
+      <ns0:c r="A8" t="inlineStr">
+        <ns0:is>
+          <ns0:t>CLAUDE-4723-O3</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B8" t="inlineStr">
+        <ns0:is>
+          <ns0:t>S1</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C8" t="inlineStr">
+        <ns0:is>
+          <ns0:t>D4-BOUNDARY-O3</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D8" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Proxy/server must withhold locked response data</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E8" t="inlineStr">
+        <ns0:is>
+          <ns0:t>CLAUDE_PRODUCT_REVIEW_4723f603 and readiness addendum</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F8" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Existing productSuccessor work item / Codex</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G8" t="inlineStr">
+        <ns0:is>
+          <ns0:t>FIXED AWAITING RETEST</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H8" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Amendment commit containing this record</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I8" t="inlineStr">
+        <ns0:is>
+          <ns0:t>CODEX_D3_D4_PRODUCT_SUCCESSOR_REVISION/REVIEW.md</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J8" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Shared Clinic / dependent controls</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K8" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Independent review and hosted acceptance not waived</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="9">
+      <ns0:c r="A9" t="inlineStr">
+        <ns0:is>
+          <ns0:t>CLAUDE-4723-O1</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B9" t="inlineStr">
+        <ns0:is>
+          <ns0:t>S2</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C9" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P10-06 instances pending</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D9" t="inlineStr">
+        <ns0:is>
+          <ns0:t>JS-enabled hydration failure needs explanatory feedback</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E9" t="inlineStr">
+        <ns0:is>
+          <ns0:t>CLAUDE_PRODUCT_REVIEW_4723f603 O1</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F9" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Existing productSuccessor work item / Codex</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G9" t="inlineStr">
+        <ns0:is>
+          <ns0:t>OPEN</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H9" t="inlineStr">
+        <ns0:is>
+          <ns0:t>4723 D3 unchanged</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I9" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Existing security evidence only</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J9" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Auth usability</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K9" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Security PASS does not waive usability, EN/ES, assistive-tech or real-device acceptance</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+  </ns0:sheetData>
+  <ns0:mergeCells>
+    <ns0:mergeCell ref="A1:K1"/>
+    <ns0:mergeCell ref="A2:K2"/>
+  </ns0:mergeCells>
+  <ns0:dataValidations count="2">
+    <ns0:dataValidation type="list" sqref="B5:B1000">
+      <ns0:formula1>"S0,S1,S2,S3"</ns0:formula1>
+    </ns0:dataValidation>
+    <ns0:dataValidation type="list" sqref="G5:G1000">
+      <ns0:formula1>"OPEN,ASSIGNED,FIXED AWAITING RETEST,CLOSED,BLOCKED"</ns0:formula1>
+    </ns0:dataValidation>
+  </ns0:dataValidations>
+  <ns0:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ns0:tableParts count="1">
+    <ns0:tablePart ns1:id="R087daac7a3394538"/>
+  </ns0:tableParts>
+</ns0:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
fix: reject invalid NY anchors and localize Nevada result
</commit_message>
<xml_diff>
--- a/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
+++ b/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
@@ -546,7 +546,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<ns0:table xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<ns0:table xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N42" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <ns0:tableColumns count="14">
     <ns0:tableColumn id="1" name="Case ID"/>
     <ns0:tableColumn id="2" name="Control ID"/>
@@ -8784,6 +8784,2454 @@
         </ns0:is>
       </ns0:c>
     </ns0:row>
+    <ns0:row r="9">
+      <ns0:c r="A9" t="inlineStr">
+        <ns0:is>
+          <ns0:t>B001-NV-automatic_discharge</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B9" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P02-06</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C9" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NV</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D9" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NV:probation-or-specialty-court-dismissal-set-aside-sealing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E9" t="inlineStr">
+        <ns0:is>
+          <ns0:t>automatic_discharge</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F9" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Public API</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G9" t="inlineStr">
+        <ns0:is>
+          <ns0:t>canonical wire</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H9" t="inlineStr">
+        <ns0:is>
+          <ns0:t>f5204e12ddb8e7445a70ef2c043dd2173e7e676e</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I9" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PASS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J9" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Runtime: expected guidance_only; observed guidance_only; HTTP 200; commercial flags held=True. Independent QA NOT RUN.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K9" t="inlineStr">
+        <ns0:is>
+          <ns0:t>/workspaces/training-modules-09-10/output/nationwide-correction-execution-20261011/checkpoints/active-assignments-20261012-v1/final-acceptance-batch-001/API-RESULTS-v1.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L9" t="inlineStr">
+        <ns0:is>
+          <ns0:t>R Codex executed; G independent QA pending; H-L qualified legal review pending</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M9" t="inlineStr">
+        <ns0:is>
+          <ns0:t>GA-42</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N9" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Only exact source-derived assertion, not complete route or delivery. EXPECTED.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="10">
+      <ns0:c r="A10" t="inlineStr">
+        <ns0:is>
+          <ns0:t>B001-NV-petition_elapsed</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B10" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P02-03</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C10" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NV</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D10" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NV:probation-or-specialty-court-dismissal-set-aside-sealing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E10" t="inlineStr">
+        <ns0:is>
+          <ns0:t>petition_elapsed</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F10" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Public API</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G10" t="inlineStr">
+        <ns0:is>
+          <ns0:t>canonical wire</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H10" t="inlineStr">
+        <ns0:is>
+          <ns0:t>f5204e12ddb8e7445a70ef2c043dd2173e7e676e</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I10" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PASS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J10" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Runtime: expected packet_ready_with_caution; observed packet_ready_with_caution; HTTP 200; commercial flags held=True. Independent QA NOT RUN.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K10" t="inlineStr">
+        <ns0:is>
+          <ns0:t>/workspaces/training-modules-09-10/output/nationwide-correction-execution-20261011/checkpoints/active-assignments-20261012-v1/final-acceptance-batch-001/API-RESULTS-v1.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L10" t="inlineStr">
+        <ns0:is>
+          <ns0:t>R Codex executed; G independent QA pending; H-L qualified legal review pending</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M10" t="inlineStr">
+        <ns0:is>
+          <ns0:t>GA-42</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N10" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Only exact source-derived assertion, not complete route or delivery. EXPECTED.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="11">
+      <ns0:c r="A11" t="inlineStr">
+        <ns0:is>
+          <ns0:t>B001-NV-petition_recent</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B11" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P02-03</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C11" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NV</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D11" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NV:probation-or-specialty-court-dismissal-set-aside-sealing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E11" t="inlineStr">
+        <ns0:is>
+          <ns0:t>petition_recent</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F11" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Public API</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G11" t="inlineStr">
+        <ns0:is>
+          <ns0:t>canonical wire</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H11" t="inlineStr">
+        <ns0:is>
+          <ns0:t>f5204e12ddb8e7445a70ef2c043dd2173e7e676e</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I11" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PASS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J11" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Runtime: expected not_yet; observed not_yet; HTTP 200; commercial flags held=True. Independent QA NOT RUN.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K11" t="inlineStr">
+        <ns0:is>
+          <ns0:t>/workspaces/training-modules-09-10/output/nationwide-correction-execution-20261011/checkpoints/active-assignments-20261012-v1/final-acceptance-batch-001/API-RESULTS-v1.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L11" t="inlineStr">
+        <ns0:is>
+          <ns0:t>R Codex executed; G independent QA pending; H-L qualified legal review pending</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M11" t="inlineStr">
+        <ns0:is>
+          <ns0:t>GA-42</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N11" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Only exact source-derived assertion, not complete route or delivery. EXPECTED.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="12">
+      <ns0:c r="A12" t="inlineStr">
+        <ns0:is>
+          <ns0:t>B001-NV-excluded_charge</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B12" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P02-03</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C12" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NV</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D12" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NV:probation-or-specialty-court-dismissal-set-aside-sealing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E12" t="inlineStr">
+        <ns0:is>
+          <ns0:t>excluded_charge</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F12" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Public API</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G12" t="inlineStr">
+        <ns0:is>
+          <ns0:t>canonical wire</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H12" t="inlineStr">
+        <ns0:is>
+          <ns0:t>f5204e12ddb8e7445a70ef2c043dd2173e7e676e</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I12" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PASS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J12" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Runtime: expected likely_not_eligible; observed likely_not_eligible; HTTP 200; commercial flags held=True. Independent QA NOT RUN.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K12" t="inlineStr">
+        <ns0:is>
+          <ns0:t>/workspaces/training-modules-09-10/output/nationwide-correction-execution-20261011/checkpoints/active-assignments-20261012-v1/final-acceptance-batch-001/API-RESULTS-v1.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L12" t="inlineStr">
+        <ns0:is>
+          <ns0:t>R Codex executed; G independent QA pending; H-L qualified legal review pending</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M12" t="inlineStr">
+        <ns0:is>
+          <ns0:t>GA-42</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N12" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Only exact source-derived assertion, not complete route or delivery. EXPECTED.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="13">
+      <ns0:c r="A13" t="inlineStr">
+        <ns0:is>
+          <ns0:t>B001-NV-unknown_disposition</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B13" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P02-05</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C13" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NV</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D13" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NV:probation-or-specialty-court-dismissal-set-aside-sealing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E13" t="inlineStr">
+        <ns0:is>
+          <ns0:t>unknown_disposition</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F13" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Public API</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G13" t="inlineStr">
+        <ns0:is>
+          <ns0:t>canonical wire</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H13" t="inlineStr">
+        <ns0:is>
+          <ns0:t>f5204e12ddb8e7445a70ef2c043dd2173e7e676e</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I13" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PASS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J13" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Runtime: expected needs_more_info; observed needs_more_info; HTTP 200; commercial flags held=True. Independent QA NOT RUN.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K13" t="inlineStr">
+        <ns0:is>
+          <ns0:t>/workspaces/training-modules-09-10/output/nationwide-correction-execution-20261011/checkpoints/active-assignments-20261012-v1/final-acceptance-batch-001/API-RESULTS-v1.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L13" t="inlineStr">
+        <ns0:is>
+          <ns0:t>R Codex executed; G independent QA pending; H-L qualified legal review pending</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M13" t="inlineStr">
+        <ns0:is>
+          <ns0:t>GA-42</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N13" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Only exact source-derived assertion, not complete route or delivery. EXPECTED.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="14">
+      <ns0:c r="A14" t="inlineStr">
+        <ns0:is>
+          <ns0:t>B001-NV-seven-year-day-before</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B14" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P02-04</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C14" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NV</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D14" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NV:probation-or-specialty-court-dismissal-set-aside-sealing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E14" t="inlineStr">
+        <ns0:is>
+          <ns0:t>boundary</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F14" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Public API</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G14" t="inlineStr">
+        <ns0:is>
+          <ns0:t>canonical wire</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H14" t="inlineStr">
+        <ns0:is>
+          <ns0:t>f5204e12ddb8e7445a70ef2c043dd2173e7e676e</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I14" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PASS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J14" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Runtime: expected not_yet; observed not_yet; HTTP 200; commercial flags held=True. Independent QA NOT RUN.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K14" t="inlineStr">
+        <ns0:is>
+          <ns0:t>/workspaces/training-modules-09-10/output/nationwide-correction-execution-20261011/checkpoints/active-assignments-20261012-v1/final-acceptance-batch-001/API-RESULTS-v1.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L14" t="inlineStr">
+        <ns0:is>
+          <ns0:t>R Codex executed; G independent QA pending; H-L qualified legal review pending</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M14" t="inlineStr">
+        <ns0:is>
+          <ns0:t>GA-42</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N14" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Only exact source-derived assertion, not complete route or delivery. EXPECTED.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="15">
+      <ns0:c r="A15" t="inlineStr">
+        <ns0:is>
+          <ns0:t>B001-NV-seven-year-anniversary</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B15" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P02-04</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C15" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NV</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D15" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NV:probation-or-specialty-court-dismissal-set-aside-sealing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E15" t="inlineStr">
+        <ns0:is>
+          <ns0:t>boundary</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F15" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Public API</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G15" t="inlineStr">
+        <ns0:is>
+          <ns0:t>canonical wire</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H15" t="inlineStr">
+        <ns0:is>
+          <ns0:t>f5204e12ddb8e7445a70ef2c043dd2173e7e676e</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I15" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PASS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J15" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Runtime: expected packet_ready_with_caution; observed packet_ready_with_caution; HTTP 200; commercial flags held=True. Independent QA NOT RUN.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K15" t="inlineStr">
+        <ns0:is>
+          <ns0:t>/workspaces/training-modules-09-10/output/nationwide-correction-execution-20261011/checkpoints/active-assignments-20261012-v1/final-acceptance-batch-001/API-RESULTS-v1.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L15" t="inlineStr">
+        <ns0:is>
+          <ns0:t>R Codex executed; G independent QA pending; H-L qualified legal review pending</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M15" t="inlineStr">
+        <ns0:is>
+          <ns0:t>GA-42</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N15" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Only exact source-derived assertion, not complete route or delivery. EXPECTED.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="16">
+      <ns0:c r="A16" t="inlineStr">
+        <ns0:is>
+          <ns0:t>B001-NV-seven-year-day-after</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B16" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P02-04</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C16" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NV</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D16" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NV:probation-or-specialty-court-dismissal-set-aside-sealing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E16" t="inlineStr">
+        <ns0:is>
+          <ns0:t>boundary</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F16" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Public API</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G16" t="inlineStr">
+        <ns0:is>
+          <ns0:t>canonical wire</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H16" t="inlineStr">
+        <ns0:is>
+          <ns0:t>f5204e12ddb8e7445a70ef2c043dd2173e7e676e</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I16" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PASS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J16" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Runtime: expected packet_ready_with_caution; observed packet_ready_with_caution; HTTP 200; commercial flags held=True. Independent QA NOT RUN.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K16" t="inlineStr">
+        <ns0:is>
+          <ns0:t>/workspaces/training-modules-09-10/output/nationwide-correction-execution-20261011/checkpoints/active-assignments-20261012-v1/final-acceptance-batch-001/API-RESULTS-v1.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L16" t="inlineStr">
+        <ns0:is>
+          <ns0:t>R Codex executed; G independent QA pending; H-L qualified legal review pending</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M16" t="inlineStr">
+        <ns0:is>
+          <ns0:t>GA-42</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N16" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Only exact source-derived assertion, not complete route or delivery. EXPECTED.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="17">
+      <ns0:c r="A17" t="inlineStr">
+        <ns0:is>
+          <ns0:t>B001-NY-positive</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B17" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P02-03</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C17" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NY</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D17" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NY:discretionary-conviction-sealing-by-petition-under-cpl-160-59</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E17" t="inlineStr">
+        <ns0:is>
+          <ns0:t>positive</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F17" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Public API</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G17" t="inlineStr">
+        <ns0:is>
+          <ns0:t>canonical wire</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H17" t="inlineStr">
+        <ns0:is>
+          <ns0:t>f5204e12ddb8e7445a70ef2c043dd2173e7e676e</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I17" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PASS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J17" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Runtime: expected packet_ready_with_caution; observed packet_ready_with_caution; HTTP 200; commercial flags held=True. Independent QA NOT RUN.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K17" t="inlineStr">
+        <ns0:is>
+          <ns0:t>/workspaces/training-modules-09-10/output/nationwide-correction-execution-20261011/checkpoints/active-assignments-20261012-v1/final-acceptance-batch-001/API-RESULTS-v1.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L17" t="inlineStr">
+        <ns0:is>
+          <ns0:t>R Codex executed; G independent QA pending; H-L qualified legal review pending</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M17" t="inlineStr">
+        <ns0:is>
+          <ns0:t>GA-19</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N17" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Only exact source-derived assertion, not complete route or delivery. EXPECTED.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="18">
+      <ns0:c r="A18" t="inlineStr">
+        <ns0:is>
+          <ns0:t>B001-NY-later-conviction</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B18" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P02-03</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C18" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NY</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D18" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NY:discretionary-conviction-sealing-by-petition-under-cpl-160-59</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E18" t="inlineStr">
+        <ns0:is>
+          <ns0:t>later-conviction</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F18" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Public API</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G18" t="inlineStr">
+        <ns0:is>
+          <ns0:t>canonical wire</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H18" t="inlineStr">
+        <ns0:is>
+          <ns0:t>f5204e12ddb8e7445a70ef2c043dd2173e7e676e</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I18" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PASS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J18" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Runtime: expected likely_not_eligible; observed likely_not_eligible; HTTP 200; commercial flags held=True. Independent QA NOT RUN.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K18" t="inlineStr">
+        <ns0:is>
+          <ns0:t>/workspaces/training-modules-09-10/output/nationwide-correction-execution-20261011/checkpoints/active-assignments-20261012-v1/final-acceptance-batch-001/API-RESULTS-v1.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L18" t="inlineStr">
+        <ns0:is>
+          <ns0:t>R Codex executed; G independent QA pending; H-L qualified legal review pending</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M18" t="inlineStr">
+        <ns0:is>
+          <ns0:t>GA-19</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N18" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Only exact source-derived assertion, not complete route or delivery. EXPECTED.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="19">
+      <ns0:c r="A19" t="inlineStr">
+        <ns0:is>
+          <ns0:t>B001-NY-later-unknown</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B19" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P02-05</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C19" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NY</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D19" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NY:discretionary-conviction-sealing-by-petition-under-cpl-160-59</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E19" t="inlineStr">
+        <ns0:is>
+          <ns0:t>later-unknown</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F19" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Public API</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G19" t="inlineStr">
+        <ns0:is>
+          <ns0:t>canonical wire</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H19" t="inlineStr">
+        <ns0:is>
+          <ns0:t>f5204e12ddb8e7445a70ef2c043dd2173e7e676e</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I19" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PASS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J19" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Runtime: expected needs_review; observed needs_review; HTTP 200; commercial flags held=True. Independent QA NOT RUN.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K19" t="inlineStr">
+        <ns0:is>
+          <ns0:t>/workspaces/training-modules-09-10/output/nationwide-correction-execution-20261011/checkpoints/active-assignments-20261012-v1/final-acceptance-batch-001/API-RESULTS-v1.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L19" t="inlineStr">
+        <ns0:is>
+          <ns0:t>R Codex executed; G independent QA pending; H-L qualified legal review pending</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M19" t="inlineStr">
+        <ns0:is>
+          <ns0:t>GA-19</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N19" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Only exact source-derived assertion, not complete route or delivery. EXPECTED.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="20">
+      <ns0:c r="A20" t="inlineStr">
+        <ns0:is>
+          <ns0:t>B001-NY-arrest</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B20" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P02-03</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C20" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NY</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D20" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NY:discretionary-conviction-sealing-by-petition-under-cpl-160-59</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E20" t="inlineStr">
+        <ns0:is>
+          <ns0:t>arrest</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F20" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Public API</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G20" t="inlineStr">
+        <ns0:is>
+          <ns0:t>canonical wire</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H20" t="inlineStr">
+        <ns0:is>
+          <ns0:t>f5204e12ddb8e7445a70ef2c043dd2173e7e676e</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I20" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PASS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J20" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Runtime: expected likely_not_eligible; observed likely_not_eligible; HTTP 200; commercial flags held=True. Independent QA NOT RUN.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K20" t="inlineStr">
+        <ns0:is>
+          <ns0:t>/workspaces/training-modules-09-10/output/nationwide-correction-execution-20261011/checkpoints/active-assignments-20261012-v1/final-acceptance-batch-001/API-RESULTS-v1.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L20" t="inlineStr">
+        <ns0:is>
+          <ns0:t>R Codex executed; G independent QA pending; H-L qualified legal review pending</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M20" t="inlineStr">
+        <ns0:is>
+          <ns0:t>GA-19</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N20" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Only exact source-derived assertion, not complete route or delivery. EXPECTED.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="21">
+      <ns0:c r="A21" t="inlineStr">
+        <ns0:is>
+          <ns0:t>B001-NY-arrest-unknown</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B21" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P02-05</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C21" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NY</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D21" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NY:discretionary-conviction-sealing-by-petition-under-cpl-160-59</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E21" t="inlineStr">
+        <ns0:is>
+          <ns0:t>arrest-unknown</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F21" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Public API</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G21" t="inlineStr">
+        <ns0:is>
+          <ns0:t>canonical wire</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H21" t="inlineStr">
+        <ns0:is>
+          <ns0:t>f5204e12ddb8e7445a70ef2c043dd2173e7e676e</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I21" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PASS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J21" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Runtime: expected needs_review; observed needs_review; HTTP 200; commercial flags held=True. Independent QA NOT RUN.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K21" t="inlineStr">
+        <ns0:is>
+          <ns0:t>/workspaces/training-modules-09-10/output/nationwide-correction-execution-20261011/checkpoints/active-assignments-20261012-v1/final-acceptance-batch-001/API-RESULTS-v1.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L21" t="inlineStr">
+        <ns0:is>
+          <ns0:t>R Codex executed; G independent QA pending; H-L qualified legal review pending</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M21" t="inlineStr">
+        <ns0:is>
+          <ns0:t>GA-19</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N21" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Only exact source-derived assertion, not complete route or delivery. EXPECTED.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="22">
+      <ns0:c r="A22" t="inlineStr">
+        <ns0:is>
+          <ns0:t>B001-NY-ten-year-before</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B22" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P02-04</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C22" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NY</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D22" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NY:discretionary-conviction-sealing-by-petition-under-cpl-160-59</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E22" t="inlineStr">
+        <ns0:is>
+          <ns0:t>ten-year-before</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F22" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Public API</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G22" t="inlineStr">
+        <ns0:is>
+          <ns0:t>canonical wire</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H22" t="inlineStr">
+        <ns0:is>
+          <ns0:t>f5204e12ddb8e7445a70ef2c043dd2173e7e676e</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I22" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PASS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J22" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Runtime: expected not_yet; observed not_yet; HTTP 200; commercial flags held=True. Independent QA NOT RUN.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K22" t="inlineStr">
+        <ns0:is>
+          <ns0:t>/workspaces/training-modules-09-10/output/nationwide-correction-execution-20261011/checkpoints/active-assignments-20261012-v1/final-acceptance-batch-001/API-RESULTS-v1.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L22" t="inlineStr">
+        <ns0:is>
+          <ns0:t>R Codex executed; G independent QA pending; H-L qualified legal review pending</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M22" t="inlineStr">
+        <ns0:is>
+          <ns0:t>GA-19</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N22" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Only exact source-derived assertion, not complete route or delivery. EXPECTED.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="23">
+      <ns0:c r="A23" t="inlineStr">
+        <ns0:is>
+          <ns0:t>B001-NY-ten-year-on</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B23" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P02-04</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C23" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NY</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D23" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NY:discretionary-conviction-sealing-by-petition-under-cpl-160-59</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E23" t="inlineStr">
+        <ns0:is>
+          <ns0:t>ten-year-on</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F23" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Public API</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G23" t="inlineStr">
+        <ns0:is>
+          <ns0:t>canonical wire</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H23" t="inlineStr">
+        <ns0:is>
+          <ns0:t>f5204e12ddb8e7445a70ef2c043dd2173e7e676e</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I23" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PASS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J23" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Runtime: expected packet_ready_with_caution; observed packet_ready_with_caution; HTTP 200; commercial flags held=True. Independent QA NOT RUN.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K23" t="inlineStr">
+        <ns0:is>
+          <ns0:t>/workspaces/training-modules-09-10/output/nationwide-correction-execution-20261011/checkpoints/active-assignments-20261012-v1/final-acceptance-batch-001/API-RESULTS-v1.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L23" t="inlineStr">
+        <ns0:is>
+          <ns0:t>R Codex executed; G independent QA pending; H-L qualified legal review pending</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M23" t="inlineStr">
+        <ns0:is>
+          <ns0:t>GA-19</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N23" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Only exact source-derived assertion, not complete route or delivery. EXPECTED.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="24">
+      <ns0:c r="A24" t="inlineStr">
+        <ns0:is>
+          <ns0:t>B001-NY-ten-year-after</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B24" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P02-04</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C24" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NY</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D24" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NY:discretionary-conviction-sealing-by-petition-under-cpl-160-59</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E24" t="inlineStr">
+        <ns0:is>
+          <ns0:t>ten-year-after</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F24" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Public API</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G24" t="inlineStr">
+        <ns0:is>
+          <ns0:t>canonical wire</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H24" t="inlineStr">
+        <ns0:is>
+          <ns0:t>f5204e12ddb8e7445a70ef2c043dd2173e7e676e</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I24" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PASS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J24" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Runtime: expected packet_ready_with_caution; observed packet_ready_with_caution; HTTP 200; commercial flags held=True. Independent QA NOT RUN.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K24" t="inlineStr">
+        <ns0:is>
+          <ns0:t>/workspaces/training-modules-09-10/output/nationwide-correction-execution-20261011/checkpoints/active-assignments-20261012-v1/final-acceptance-batch-001/API-RESULTS-v1.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L24" t="inlineStr">
+        <ns0:is>
+          <ns0:t>R Codex executed; G independent QA pending; H-L qualified legal review pending</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M24" t="inlineStr">
+        <ns0:is>
+          <ns0:t>GA-19</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N24" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Only exact source-derived assertion, not complete route or delivery. EXPECTED.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="25">
+      <ns0:c r="A25" t="inlineStr">
+        <ns0:is>
+          <ns0:t>B001-NY-invalid-calendar</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B25" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P02-04</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C25" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NY</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D25" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NY:discretionary-conviction-sealing-by-petition-under-cpl-160-59</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E25" t="inlineStr">
+        <ns0:is>
+          <ns0:t>invalid-calendar</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F25" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Public API</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G25" t="inlineStr">
+        <ns0:is>
+          <ns0:t>canonical wire</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H25" t="inlineStr">
+        <ns0:is>
+          <ns0:t>f5204e12ddb8e7445a70ef2c043dd2173e7e676e</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I25" t="inlineStr">
+        <ns0:is>
+          <ns0:t>FAIL</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J25" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Runtime: expected needs_more_info; observed packet_ready_with_caution; HTTP 200; commercial flags held=True. Independent QA NOT RUN.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K25" t="inlineStr">
+        <ns0:is>
+          <ns0:t>/workspaces/training-modules-09-10/output/nationwide-correction-execution-20261011/checkpoints/active-assignments-20261012-v1/final-acceptance-batch-001/API-RESULTS-v1.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L25" t="inlineStr">
+        <ns0:is>
+          <ns0:t>R Codex executed; G independent QA pending; H-L qualified legal review pending</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M25" t="inlineStr">
+        <ns0:is>
+          <ns0:t>GA-19</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N25" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Only exact source-derived assertion, not complete route or delivery. EXPECTED.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="26">
+      <ns0:c r="A26" t="inlineStr">
+        <ns0:is>
+          <ns0:t>B001-NY-positive-retest</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B26" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P02-03</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C26" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NY</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D26" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NY:discretionary-conviction-sealing-by-petition-under-cpl-160-59</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E26" t="inlineStr">
+        <ns0:is>
+          <ns0:t>positive</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F26" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Public API</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G26" t="inlineStr">
+        <ns0:is>
+          <ns0:t>canonical wire</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H26" t="inlineStr">
+        <ns0:is>
+          <ns0:t>f5204e12d + atomic source hashes in ATOMIC-CORRECTION.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I26" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PASS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J26" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Runtime: expected packet_ready_with_caution; observed packet_ready_with_caution; HTTP 200; commercial flags held=True. Independent QA NOT RUN.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K26" t="inlineStr">
+        <ns0:is>
+          <ns0:t>/workspaces/training-modules-09-10/output/nationwide-correction-execution-20261011/checkpoints/active-assignments-20261012-v1/final-acceptance-batch-001/API-RESULTS-correction-v2.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L26" t="inlineStr">
+        <ns0:is>
+          <ns0:t>R Codex executed; G independent QA pending; H-L qualified legal review pending</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M26" t="inlineStr">
+        <ns0:is>
+          <ns0:t>GA-19</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N26" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Only exact source-derived assertion, not complete route or delivery. EXPECTED.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="27">
+      <ns0:c r="A27" t="inlineStr">
+        <ns0:is>
+          <ns0:t>B001-NY-later-conviction-retest</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B27" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P02-03</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C27" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NY</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D27" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NY:discretionary-conviction-sealing-by-petition-under-cpl-160-59</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E27" t="inlineStr">
+        <ns0:is>
+          <ns0:t>later-conviction</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F27" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Public API</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G27" t="inlineStr">
+        <ns0:is>
+          <ns0:t>canonical wire</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H27" t="inlineStr">
+        <ns0:is>
+          <ns0:t>f5204e12d + atomic source hashes in ATOMIC-CORRECTION.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I27" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PASS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J27" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Runtime: expected likely_not_eligible; observed likely_not_eligible; HTTP 200; commercial flags held=True. Independent QA NOT RUN.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K27" t="inlineStr">
+        <ns0:is>
+          <ns0:t>/workspaces/training-modules-09-10/output/nationwide-correction-execution-20261011/checkpoints/active-assignments-20261012-v1/final-acceptance-batch-001/API-RESULTS-correction-v2.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L27" t="inlineStr">
+        <ns0:is>
+          <ns0:t>R Codex executed; G independent QA pending; H-L qualified legal review pending</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M27" t="inlineStr">
+        <ns0:is>
+          <ns0:t>GA-19</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N27" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Only exact source-derived assertion, not complete route or delivery. EXPECTED.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="28">
+      <ns0:c r="A28" t="inlineStr">
+        <ns0:is>
+          <ns0:t>B001-NY-later-unknown-retest</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B28" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P02-05</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C28" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NY</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D28" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NY:discretionary-conviction-sealing-by-petition-under-cpl-160-59</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E28" t="inlineStr">
+        <ns0:is>
+          <ns0:t>later-unknown</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F28" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Public API</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G28" t="inlineStr">
+        <ns0:is>
+          <ns0:t>canonical wire</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H28" t="inlineStr">
+        <ns0:is>
+          <ns0:t>f5204e12d + atomic source hashes in ATOMIC-CORRECTION.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I28" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PASS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J28" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Runtime: expected needs_review; observed needs_review; HTTP 200; commercial flags held=True. Independent QA NOT RUN.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K28" t="inlineStr">
+        <ns0:is>
+          <ns0:t>/workspaces/training-modules-09-10/output/nationwide-correction-execution-20261011/checkpoints/active-assignments-20261012-v1/final-acceptance-batch-001/API-RESULTS-correction-v2.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L28" t="inlineStr">
+        <ns0:is>
+          <ns0:t>R Codex executed; G independent QA pending; H-L qualified legal review pending</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M28" t="inlineStr">
+        <ns0:is>
+          <ns0:t>GA-19</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N28" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Only exact source-derived assertion, not complete route or delivery. EXPECTED.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="29">
+      <ns0:c r="A29" t="inlineStr">
+        <ns0:is>
+          <ns0:t>B001-NY-arrest-retest</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B29" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P02-03</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C29" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NY</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D29" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NY:discretionary-conviction-sealing-by-petition-under-cpl-160-59</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E29" t="inlineStr">
+        <ns0:is>
+          <ns0:t>arrest</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F29" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Public API</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G29" t="inlineStr">
+        <ns0:is>
+          <ns0:t>canonical wire</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H29" t="inlineStr">
+        <ns0:is>
+          <ns0:t>f5204e12d + atomic source hashes in ATOMIC-CORRECTION.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I29" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PASS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J29" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Runtime: expected likely_not_eligible; observed likely_not_eligible; HTTP 200; commercial flags held=True. Independent QA NOT RUN.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K29" t="inlineStr">
+        <ns0:is>
+          <ns0:t>/workspaces/training-modules-09-10/output/nationwide-correction-execution-20261011/checkpoints/active-assignments-20261012-v1/final-acceptance-batch-001/API-RESULTS-correction-v2.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L29" t="inlineStr">
+        <ns0:is>
+          <ns0:t>R Codex executed; G independent QA pending; H-L qualified legal review pending</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M29" t="inlineStr">
+        <ns0:is>
+          <ns0:t>GA-19</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N29" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Only exact source-derived assertion, not complete route or delivery. EXPECTED.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="30">
+      <ns0:c r="A30" t="inlineStr">
+        <ns0:is>
+          <ns0:t>B001-NY-arrest-unknown-retest</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B30" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P02-05</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C30" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NY</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D30" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NY:discretionary-conviction-sealing-by-petition-under-cpl-160-59</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E30" t="inlineStr">
+        <ns0:is>
+          <ns0:t>arrest-unknown</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F30" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Public API</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G30" t="inlineStr">
+        <ns0:is>
+          <ns0:t>canonical wire</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H30" t="inlineStr">
+        <ns0:is>
+          <ns0:t>f5204e12d + atomic source hashes in ATOMIC-CORRECTION.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I30" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PASS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J30" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Runtime: expected needs_review; observed needs_review; HTTP 200; commercial flags held=True. Independent QA NOT RUN.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K30" t="inlineStr">
+        <ns0:is>
+          <ns0:t>/workspaces/training-modules-09-10/output/nationwide-correction-execution-20261011/checkpoints/active-assignments-20261012-v1/final-acceptance-batch-001/API-RESULTS-correction-v2.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L30" t="inlineStr">
+        <ns0:is>
+          <ns0:t>R Codex executed; G independent QA pending; H-L qualified legal review pending</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M30" t="inlineStr">
+        <ns0:is>
+          <ns0:t>GA-19</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N30" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Only exact source-derived assertion, not complete route or delivery. EXPECTED.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="31">
+      <ns0:c r="A31" t="inlineStr">
+        <ns0:is>
+          <ns0:t>B001-NY-ten-year-before-retest</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B31" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P02-04</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C31" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NY</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D31" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NY:discretionary-conviction-sealing-by-petition-under-cpl-160-59</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E31" t="inlineStr">
+        <ns0:is>
+          <ns0:t>ten-year-before</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F31" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Public API</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G31" t="inlineStr">
+        <ns0:is>
+          <ns0:t>canonical wire</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H31" t="inlineStr">
+        <ns0:is>
+          <ns0:t>f5204e12d + atomic source hashes in ATOMIC-CORRECTION.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I31" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PASS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J31" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Runtime: expected not_yet; observed not_yet; HTTP 200; commercial flags held=True. Independent QA NOT RUN.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K31" t="inlineStr">
+        <ns0:is>
+          <ns0:t>/workspaces/training-modules-09-10/output/nationwide-correction-execution-20261011/checkpoints/active-assignments-20261012-v1/final-acceptance-batch-001/API-RESULTS-correction-v2.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L31" t="inlineStr">
+        <ns0:is>
+          <ns0:t>R Codex executed; G independent QA pending; H-L qualified legal review pending</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M31" t="inlineStr">
+        <ns0:is>
+          <ns0:t>GA-19</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N31" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Only exact source-derived assertion, not complete route or delivery. EXPECTED.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="32">
+      <ns0:c r="A32" t="inlineStr">
+        <ns0:is>
+          <ns0:t>B001-NY-ten-year-on-retest</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B32" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P02-04</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C32" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NY</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D32" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NY:discretionary-conviction-sealing-by-petition-under-cpl-160-59</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E32" t="inlineStr">
+        <ns0:is>
+          <ns0:t>ten-year-on</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F32" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Public API</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G32" t="inlineStr">
+        <ns0:is>
+          <ns0:t>canonical wire</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H32" t="inlineStr">
+        <ns0:is>
+          <ns0:t>f5204e12d + atomic source hashes in ATOMIC-CORRECTION.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I32" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PASS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J32" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Runtime: expected packet_ready_with_caution; observed packet_ready_with_caution; HTTP 200; commercial flags held=True. Independent QA NOT RUN.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K32" t="inlineStr">
+        <ns0:is>
+          <ns0:t>/workspaces/training-modules-09-10/output/nationwide-correction-execution-20261011/checkpoints/active-assignments-20261012-v1/final-acceptance-batch-001/API-RESULTS-correction-v2.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L32" t="inlineStr">
+        <ns0:is>
+          <ns0:t>R Codex executed; G independent QA pending; H-L qualified legal review pending</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M32" t="inlineStr">
+        <ns0:is>
+          <ns0:t>GA-19</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N32" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Only exact source-derived assertion, not complete route or delivery. EXPECTED.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="33">
+      <ns0:c r="A33" t="inlineStr">
+        <ns0:is>
+          <ns0:t>B001-NY-ten-year-after-retest</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B33" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P02-04</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C33" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NY</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D33" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NY:discretionary-conviction-sealing-by-petition-under-cpl-160-59</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E33" t="inlineStr">
+        <ns0:is>
+          <ns0:t>ten-year-after</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F33" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Public API</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G33" t="inlineStr">
+        <ns0:is>
+          <ns0:t>canonical wire</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H33" t="inlineStr">
+        <ns0:is>
+          <ns0:t>f5204e12d + atomic source hashes in ATOMIC-CORRECTION.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I33" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PASS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J33" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Runtime: expected packet_ready_with_caution; observed packet_ready_with_caution; HTTP 200; commercial flags held=True. Independent QA NOT RUN.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K33" t="inlineStr">
+        <ns0:is>
+          <ns0:t>/workspaces/training-modules-09-10/output/nationwide-correction-execution-20261011/checkpoints/active-assignments-20261012-v1/final-acceptance-batch-001/API-RESULTS-correction-v2.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L33" t="inlineStr">
+        <ns0:is>
+          <ns0:t>R Codex executed; G independent QA pending; H-L qualified legal review pending</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M33" t="inlineStr">
+        <ns0:is>
+          <ns0:t>GA-19</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N33" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Only exact source-derived assertion, not complete route or delivery. EXPECTED.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="34">
+      <ns0:c r="A34" t="inlineStr">
+        <ns0:is>
+          <ns0:t>B001-NY-invalid-calendar-retest</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B34" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P02-04</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C34" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NY</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D34" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NY:discretionary-conviction-sealing-by-petition-under-cpl-160-59</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E34" t="inlineStr">
+        <ns0:is>
+          <ns0:t>invalid-calendar</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F34" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Public API</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G34" t="inlineStr">
+        <ns0:is>
+          <ns0:t>canonical wire</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H34" t="inlineStr">
+        <ns0:is>
+          <ns0:t>f5204e12d + atomic source hashes in ATOMIC-CORRECTION.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I34" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PASS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J34" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Runtime: expected needs_more_info; observed needs_more_info; HTTP 200; commercial flags held=True. Independent QA NOT RUN.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K34" t="inlineStr">
+        <ns0:is>
+          <ns0:t>/workspaces/training-modules-09-10/output/nationwide-correction-execution-20261011/checkpoints/active-assignments-20261012-v1/final-acceptance-batch-001/API-RESULTS-correction-v2.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L34" t="inlineStr">
+        <ns0:is>
+          <ns0:t>R Codex executed; G independent QA pending; H-L qualified legal review pending</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M34" t="inlineStr">
+        <ns0:is>
+          <ns0:t>GA-19</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N34" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Only exact source-derived assertion, not complete route or delivery. EXPECTED.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="35">
+      <ns0:c r="A35" t="inlineStr">
+        <ns0:is>
+          <ns0:t>B001-UI-NV-en-automatic_discharge</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B35" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P03-21</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C35" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NV</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D35" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NV:probation-or-specialty-court-dismissal-set-aside-sealing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E35" t="inlineStr">
+        <ns0:is>
+          <ns0:t>automatic_discharge</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F35" t="inlineStr">
+        <ns0:is>
+          <ns0:t>DTC anonymous</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G35" t="inlineStr">
+        <ns0:is>
+          <ns0:t>EN</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H35" t="inlineStr">
+        <ns0:is>
+          <ns0:t>f5204e12d</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I35" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PASS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J35" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Actual12question browser journey to result; Expected outcome and commercial hold observed; screenshot inspected by executor. Independent QA and bilingual review pending.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K35" t="inlineStr">
+        <ns0:is>
+          <ns0:t>/workspaces/training-modules-09-10/output/nationwide-correction-execution-20261011/checkpoints/active-assignments-20261012-v1/final-acceptance-batch-001/browser-v1/RESULTS.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L35" t="inlineStr">
+        <ns0:is>
+          <ns0:t>R Codex executed; G/H-A pending</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M35" t="inlineStr">
+        <ns0:is>
+          <ns0:t>GA-24;GA-42</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N35" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Browser uses broad time bucket; exact anniversary proof is separate API evidence. No protected claim, funding or delivery.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="36">
+      <ns0:c r="A36" t="inlineStr">
+        <ns0:is>
+          <ns0:t>B001-UI-NV-en-petition_elapsed</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B36" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P03-21</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C36" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NV</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D36" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NV:probation-or-specialty-court-dismissal-set-aside-sealing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E36" t="inlineStr">
+        <ns0:is>
+          <ns0:t>petition_elapsed</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F36" t="inlineStr">
+        <ns0:is>
+          <ns0:t>DTC anonymous</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G36" t="inlineStr">
+        <ns0:is>
+          <ns0:t>EN</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H36" t="inlineStr">
+        <ns0:is>
+          <ns0:t>f5204e12d</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I36" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PASS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J36" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Actual12question browser journey to result; Expected outcome and commercial hold observed; screenshot inspected by executor. Independent QA and bilingual review pending.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K36" t="inlineStr">
+        <ns0:is>
+          <ns0:t>/workspaces/training-modules-09-10/output/nationwide-correction-execution-20261011/checkpoints/active-assignments-20261012-v1/final-acceptance-batch-001/browser-v1/RESULTS.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L36" t="inlineStr">
+        <ns0:is>
+          <ns0:t>R Codex executed; G/H-A pending</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M36" t="inlineStr">
+        <ns0:is>
+          <ns0:t>GA-24;GA-42</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N36" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Browser uses broad time bucket; exact anniversary proof is separate API evidence. No protected claim, funding or delivery.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="37">
+      <ns0:c r="A37" t="inlineStr">
+        <ns0:is>
+          <ns0:t>B001-UI-NV-es-automatic_discharge</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B37" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P03-21</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C37" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NV</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D37" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NV:probation-or-specialty-court-dismissal-set-aside-sealing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E37" t="inlineStr">
+        <ns0:is>
+          <ns0:t>automatic_discharge</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F37" t="inlineStr">
+        <ns0:is>
+          <ns0:t>DTC anonymous</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G37" t="inlineStr">
+        <ns0:is>
+          <ns0:t>ES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H37" t="inlineStr">
+        <ns0:is>
+          <ns0:t>f5204e12d</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I37" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PASS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J37" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Actual12question browser journey to result; Expected outcome and commercial hold observed; screenshot inspected by executor. Independent QA and bilingual review pending.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K37" t="inlineStr">
+        <ns0:is>
+          <ns0:t>/workspaces/training-modules-09-10/output/nationwide-correction-execution-20261011/checkpoints/active-assignments-20261012-v1/final-acceptance-batch-001/browser-v1/RESULTS.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L37" t="inlineStr">
+        <ns0:is>
+          <ns0:t>R Codex executed; G/H-A pending</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M37" t="inlineStr">
+        <ns0:is>
+          <ns0:t>GA-24;GA-42</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N37" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Browser uses broad time bucket; exact anniversary proof is separate API evidence. No protected claim, funding or delivery.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="38">
+      <ns0:c r="A38" t="inlineStr">
+        <ns0:is>
+          <ns0:t>B001-UI-NV-es-petition_elapsed</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B38" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P03-21</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C38" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NV</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D38" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NV:probation-or-specialty-court-dismissal-set-aside-sealing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E38" t="inlineStr">
+        <ns0:is>
+          <ns0:t>petition_elapsed</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F38" t="inlineStr">
+        <ns0:is>
+          <ns0:t>DTC anonymous</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G38" t="inlineStr">
+        <ns0:is>
+          <ns0:t>ES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H38" t="inlineStr">
+        <ns0:is>
+          <ns0:t>f5204e12d</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I38" t="inlineStr">
+        <ns0:is>
+          <ns0:t>FAIL</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J38" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Actual12question browser journey to result; English fallback reproduced. Independent QA and bilingual review pending.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K38" t="inlineStr">
+        <ns0:is>
+          <ns0:t>/workspaces/training-modules-09-10/output/nationwide-correction-execution-20261011/checkpoints/active-assignments-20261012-v1/final-acceptance-batch-001/browser-v1/RESULTS.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L38" t="inlineStr">
+        <ns0:is>
+          <ns0:t>R Codex executed; G/H-A pending</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M38" t="inlineStr">
+        <ns0:is>
+          <ns0:t>GA-24;GA-42</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N38" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Browser uses broad time bucket; exact anniversary proof is separate API evidence. No protected claim, funding or delivery.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="39">
+      <ns0:c r="A39" t="inlineStr">
+        <ns0:is>
+          <ns0:t>B001-UI-NV-es-petition_elapsed-retest</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B39" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P03-21</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C39" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NV</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D39" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NV:probation-or-specialty-court-dismissal-set-aside-sealing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E39" t="inlineStr">
+        <ns0:is>
+          <ns0:t>petition_elapsed</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F39" t="inlineStr">
+        <ns0:is>
+          <ns0:t>DTC anonymous</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G39" t="inlineStr">
+        <ns0:is>
+          <ns0:t>ES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H39" t="inlineStr">
+        <ns0:is>
+          <ns0:t>f5204e12d + atomic source hashes in ATOMIC-CORRECTION.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I39" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PASS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J39" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Actual12question browser journey to result; Expected outcome and commercial hold observed; screenshot inspected by executor. Independent QA and bilingual review pending.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K39" t="inlineStr">
+        <ns0:is>
+          <ns0:t>/workspaces/training-modules-09-10/output/nationwide-correction-execution-20261011/checkpoints/active-assignments-20261012-v1/final-acceptance-batch-001/browser-correction-v2/RESULTS.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L39" t="inlineStr">
+        <ns0:is>
+          <ns0:t>R Codex executed; G/H-A pending</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M39" t="inlineStr">
+        <ns0:is>
+          <ns0:t>GA-24;GA-42</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N39" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Browser uses broad time bucket; exact anniversary proof is separate API evidence. No protected claim, funding or delivery.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="40">
+      <ns0:c r="A40" t="inlineStr">
+        <ns0:is>
+          <ns0:t>B001-PROTECTED-owner</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B40" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P09-02</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C40" t="inlineStr">
+        <ns0:is>
+          <ns0:t>MS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D40" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Retained isolated synthetic MS matter</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E40" t="inlineStr">
+        <ns0:is>
+          <ns0:t>owner200/staff404/anonymous401</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F40" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Protected Briefcase</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G40" t="inlineStr">
+        <ns0:is>
+          <ns0:t>EN</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H40" t="inlineStr">
+        <ns0:is>
+          <ns0:t>f5204e12d</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I40" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PASS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J40" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Actual HTTP200; ordinary sign-in=True; owner UI=True; Briefcase row unchanged. Not full journey.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K40" t="inlineStr">
+        <ns0:is>
+          <ns0:t>/workspaces/training-modules-09-10/output/nationwide-correction-execution-20261011/checkpoints/active-assignments-20261012-v1/final-acceptance-batch-001/PROTECTED-v1.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L40" t="inlineStr">
+        <ns0:is>
+          <ns0:t>R Codex executed; G independent QA pending</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M40" t="inlineStr">
+        <ns0:is>
+          <ns0:t>GA-43</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N40" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Existing authorized local identities; does not replace GA22 exact hosted Mississippi account.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="41">
+      <ns0:c r="A41" t="inlineStr">
+        <ns0:is>
+          <ns0:t>B001-PROTECTED-staff</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B41" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P09-02</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C41" t="inlineStr">
+        <ns0:is>
+          <ns0:t>MS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D41" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Retained isolated synthetic MS matter</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E41" t="inlineStr">
+        <ns0:is>
+          <ns0:t>owner200/staff404/anonymous401</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F41" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Protected Briefcase</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G41" t="inlineStr">
+        <ns0:is>
+          <ns0:t>EN</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H41" t="inlineStr">
+        <ns0:is>
+          <ns0:t>f5204e12d</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I41" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PASS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J41" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Actual HTTP404; ordinary sign-in=True; owner UI=False; Briefcase row unchanged. Not full journey.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K41" t="inlineStr">
+        <ns0:is>
+          <ns0:t>/workspaces/training-modules-09-10/output/nationwide-correction-execution-20261011/checkpoints/active-assignments-20261012-v1/final-acceptance-batch-001/PROTECTED-v1.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L41" t="inlineStr">
+        <ns0:is>
+          <ns0:t>R Codex executed; G independent QA pending</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M41" t="inlineStr">
+        <ns0:is>
+          <ns0:t>GA-43</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N41" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Existing authorized local identities; does not replace GA22 exact hosted Mississippi account.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="42">
+      <ns0:c r="A42" t="inlineStr">
+        <ns0:is>
+          <ns0:t>B001-PROTECTED-anonymous</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B42" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P09-02</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C42" t="inlineStr">
+        <ns0:is>
+          <ns0:t>MS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D42" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Retained isolated synthetic MS matter</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E42" t="inlineStr">
+        <ns0:is>
+          <ns0:t>owner200/staff404/anonymous401</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F42" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Protected Briefcase</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G42" t="inlineStr">
+        <ns0:is>
+          <ns0:t>EN</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H42" t="inlineStr">
+        <ns0:is>
+          <ns0:t>f5204e12d</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I42" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PASS</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J42" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Actual HTTP401; ordinary sign-in=False; owner UI=False; Briefcase row unchanged. Not full journey.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K42" t="inlineStr">
+        <ns0:is>
+          <ns0:t>/workspaces/training-modules-09-10/output/nationwide-correction-execution-20261011/checkpoints/active-assignments-20261012-v1/final-acceptance-batch-001/PROTECTED-v1.json</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L42" t="inlineStr">
+        <ns0:is>
+          <ns0:t>R Codex executed; G independent QA pending</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M42" t="inlineStr">
+        <ns0:is>
+          <ns0:t>GA-43</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N42" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Existing authorized local identities; does not replace GA22 exact hosted Mississippi account.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
   </ns0:sheetData>
   <ns0:mergeCells>
     <ns0:mergeCell ref="A1:N1"/>

</xml_diff>

<commit_message>
Use factual California Prop64 predicates and preserve protected corrections
</commit_message>
<xml_diff>
--- a/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
+++ b/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
@@ -24633,6 +24633,582 @@
         </x:is>
       </x:c>
     </x:row>
+    <x:row r="229">
+      <x:c r="A229" t="inlineStr">
+        <x:is>
+          <x:t>CA-PROP64-PERSISTENCE-currently-serving-petition-20261013</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B229" t="inlineStr">
+        <x:is>
+          <x:t>P03-18</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C229" t="inlineStr">
+        <x:is>
+          <x:t>CA</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D229" t="inlineStr">
+        <x:is>
+          <x:t>CA:prop-64-currently-serving-petition-11361-8</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E229" t="inlineStr">
+        <x:is>
+          <x:t>Local ordinary-owner claim/reload; held correction; actual decimal save; CAS; verify/invalidate/recover; wrong-owner denial</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F229" t="inlineStr">
+        <x:is>
+          <x:t>DTC</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G229" t="inlineStr">
+        <x:is>
+          <x:t>BOTH</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H229" t="inlineStr">
+        <x:is>
+          <x:t>Commit containing this checkpoint; PROTECTED-v6 runtime manifest</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I229" t="inlineStr">
+        <x:is>
+          <x:t>PASS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J229" t="inlineStr">
+        <x:is>
+          <x:t>53 checks across both routes; exact3-table restoration. No hosted or full-route acceptance.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K229" t="inlineStr">
+        <x:is>
+          <x:t>/workspaces/training-modules-09-10/output/nationwide-correction-execution-20261011/checkpoints/active-assignments-20261012-v1/ca-prop64-facts-20261012/PROTECTED-v7.json</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L229" t="inlineStr">
+        <x:is>
+          <x:t>Codex executed; independent engineering receipt review; qualified QA pending</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M229" t="inlineStr">
+        <x:is>
+          <x:t>GA-19 / GA-21 / GA-43 / GA-44</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N229" t="inlineStr">
+        <x:is>
+          <x:t>No payment/sponsorship/download/legal/language approval.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="230">
+      <x:c r="A230" t="inlineStr">
+        <x:is>
+          <x:t>CA-PROP64-PERSISTENCE-completed-sentence-application-20261013</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B230" t="inlineStr">
+        <x:is>
+          <x:t>P03-18</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C230" t="inlineStr">
+        <x:is>
+          <x:t>CA</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D230" t="inlineStr">
+        <x:is>
+          <x:t>CA:prop-64-completed-sentence-application-11361-8</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E230" t="inlineStr">
+        <x:is>
+          <x:t>Local ordinary-owner claim/reload; held correction; actual decimal save; CAS; verify/invalidate/recover; wrong-owner denial</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F230" t="inlineStr">
+        <x:is>
+          <x:t>DTC</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G230" t="inlineStr">
+        <x:is>
+          <x:t>BOTH</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H230" t="inlineStr">
+        <x:is>
+          <x:t>Commit containing this checkpoint; PROTECTED-v6 runtime manifest</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I230" t="inlineStr">
+        <x:is>
+          <x:t>PASS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J230" t="inlineStr">
+        <x:is>
+          <x:t>53 checks across both routes; exact3-table restoration. No hosted or full-route acceptance.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K230" t="inlineStr">
+        <x:is>
+          <x:t>/workspaces/training-modules-09-10/output/nationwide-correction-execution-20261011/checkpoints/active-assignments-20261012-v1/ca-prop64-facts-20261012/PROTECTED-v7.json</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L230" t="inlineStr">
+        <x:is>
+          <x:t>Codex executed; independent engineering receipt review; qualified QA pending</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M230" t="inlineStr">
+        <x:is>
+          <x:t>GA-19 / GA-21 / GA-43 / GA-44</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N230" t="inlineStr">
+        <x:is>
+          <x:t>No payment/sponsorship/download/legal/language approval.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="231">
+      <x:c r="A231" t="inlineStr">
+        <x:is>
+          <x:t>CA-PROP64-CA-L01-20261013</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B231" t="inlineStr">
+        <x:is>
+          <x:t>P02-05</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C231" t="inlineStr">
+        <x:is>
+          <x:t>CA</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D231" t="inlineStr">
+        <x:is>
+          <x:t>Both existing Prop64 routes</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E231" t="inlineStr">
+        <x:is>
+          <x:t>Historical concentrate/subsection interpretation</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F231" t="inlineStr">
+        <x:is>
+          <x:t>Shared</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G231" t="inlineStr">
+        <x:is>
+          <x:t>BOTH</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H231" t="inlineStr">
+        <x:is>
+          <x:t>Current candidate and existing review report</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I231" t="inlineStr">
+        <x:is>
+          <x:t>NOT RUN</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J231" t="inlineStr">
+        <x:is>
+          <x:t>Qualified decision plus dependent engineering/output/journey acceptance remains active</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K231" t="inlineStr">
+        <x:is>
+          <x:t>docs/rcap/grade-a/handoffs/NATIONWIDE_BLOCKER_RESOLUTION_INPUTS_2026-10-12.md</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L231" t="inlineStr">
+        <x:is>
+          <x:t>Codex engineering; qualified CA reviewer and independent QA</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M231" t="inlineStr">
+        <x:is>
+          <x:t>GA-19 / GA-21 / GA-49</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N231" t="inlineStr">
+        <x:is>
+          <x:t>Precise review matrix; no final disposition or fabricated approval.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="232">
+      <x:c r="A232" t="inlineStr">
+        <x:is>
+          <x:t>CA-PROP64-CA-L02-20261013</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B232" t="inlineStr">
+        <x:is>
+          <x:t>P02-05</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C232" t="inlineStr">
+        <x:is>
+          <x:t>CA</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D232" t="inlineStr">
+        <x:is>
+          <x:t>Both existing Prop64 routes</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E232" t="inlineStr">
+        <x:is>
+          <x:t>11360 conduct and exception interaction</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F232" t="inlineStr">
+        <x:is>
+          <x:t>Shared</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G232" t="inlineStr">
+        <x:is>
+          <x:t>BOTH</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H232" t="inlineStr">
+        <x:is>
+          <x:t>Current candidate and existing review report</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I232" t="inlineStr">
+        <x:is>
+          <x:t>NOT RUN</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J232" t="inlineStr">
+        <x:is>
+          <x:t>Qualified decision plus dependent engineering/output/journey acceptance remains active</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K232" t="inlineStr">
+        <x:is>
+          <x:t>docs/rcap/grade-a/handoffs/NATIONWIDE_BLOCKER_RESOLUTION_INPUTS_2026-10-12.md</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L232" t="inlineStr">
+        <x:is>
+          <x:t>Codex engineering; qualified CA reviewer and independent QA</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M232" t="inlineStr">
+        <x:is>
+          <x:t>GA-19 / GA-21 / GA-49</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N232" t="inlineStr">
+        <x:is>
+          <x:t>Precise review matrix; no final disposition or fabricated approval.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="233">
+      <x:c r="A233" t="inlineStr">
+        <x:is>
+          <x:t>CA-PROP64-CA-L03-20261013</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B233" t="inlineStr">
+        <x:is>
+          <x:t>P02-05</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C233" t="inlineStr">
+        <x:is>
+          <x:t>CA</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D233" t="inlineStr">
+        <x:is>
+          <x:t>Both existing Prop64 routes</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E233" t="inlineStr">
+        <x:is>
+          <x:t>Additional benefit after existing relief</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F233" t="inlineStr">
+        <x:is>
+          <x:t>Shared</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G233" t="inlineStr">
+        <x:is>
+          <x:t>BOTH</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H233" t="inlineStr">
+        <x:is>
+          <x:t>Current candidate and existing review report</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I233" t="inlineStr">
+        <x:is>
+          <x:t>NOT RUN</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J233" t="inlineStr">
+        <x:is>
+          <x:t>Qualified decision plus dependent engineering/output/journey acceptance remains active</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K233" t="inlineStr">
+        <x:is>
+          <x:t>docs/rcap/grade-a/handoffs/NATIONWIDE_BLOCKER_RESOLUTION_INPUTS_2026-10-12.md</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L233" t="inlineStr">
+        <x:is>
+          <x:t>Codex engineering; qualified CA reviewer and independent QA</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M233" t="inlineStr">
+        <x:is>
+          <x:t>GA-19 / GA-21 / GA-49</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N233" t="inlineStr">
+        <x:is>
+          <x:t>Precise review matrix; no final disposition or fabricated approval.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="234">
+      <x:c r="A234" t="inlineStr">
+        <x:is>
+          <x:t>CA-PROP64-CA-L04-20261013</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B234" t="inlineStr">
+        <x:is>
+          <x:t>P02-05</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C234" t="inlineStr">
+        <x:is>
+          <x:t>CA</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D234" t="inlineStr">
+        <x:is>
+          <x:t>Both existing Prop64 routes</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E234" t="inlineStr">
+        <x:is>
+          <x:t>Juvenile procedure/forms</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F234" t="inlineStr">
+        <x:is>
+          <x:t>Shared</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G234" t="inlineStr">
+        <x:is>
+          <x:t>BOTH</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H234" t="inlineStr">
+        <x:is>
+          <x:t>Current candidate and existing review report</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I234" t="inlineStr">
+        <x:is>
+          <x:t>NOT RUN</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J234" t="inlineStr">
+        <x:is>
+          <x:t>Qualified decision plus dependent engineering/output/journey acceptance remains active</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K234" t="inlineStr">
+        <x:is>
+          <x:t>docs/rcap/grade-a/handoffs/NATIONWIDE_BLOCKER_RESOLUTION_INPUTS_2026-10-12.md</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L234" t="inlineStr">
+        <x:is>
+          <x:t>Codex engineering; qualified CA reviewer and independent QA</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M234" t="inlineStr">
+        <x:is>
+          <x:t>GA-19 / GA-21 / GA-49</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N234" t="inlineStr">
+        <x:is>
+          <x:t>Precise review matrix; no final disposition or fabricated approval.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="235">
+      <x:c r="A235" t="inlineStr">
+        <x:is>
+          <x:t>CA-PROP64-CA-L05-20261013</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B235" t="inlineStr">
+        <x:is>
+          <x:t>P02-05</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C235" t="inlineStr">
+        <x:is>
+          <x:t>CA</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D235" t="inlineStr">
+        <x:is>
+          <x:t>Both existing Prop64 routes</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E235" t="inlineStr">
+        <x:is>
+          <x:t>Distinct restricted conduct and medical predicates</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F235" t="inlineStr">
+        <x:is>
+          <x:t>Shared</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G235" t="inlineStr">
+        <x:is>
+          <x:t>BOTH</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H235" t="inlineStr">
+        <x:is>
+          <x:t>Current candidate and existing review report</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I235" t="inlineStr">
+        <x:is>
+          <x:t>NOT RUN</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J235" t="inlineStr">
+        <x:is>
+          <x:t>Qualified decision plus dependent engineering/output/journey acceptance remains active</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K235" t="inlineStr">
+        <x:is>
+          <x:t>docs/rcap/grade-a/handoffs/NATIONWIDE_BLOCKER_RESOLUTION_INPUTS_2026-10-12.md</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L235" t="inlineStr">
+        <x:is>
+          <x:t>Codex engineering; qualified CA reviewer and independent QA</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M235" t="inlineStr">
+        <x:is>
+          <x:t>GA-19 / GA-21 / GA-49</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N235" t="inlineStr">
+        <x:is>
+          <x:t>Precise review matrix; no final disposition or fabricated approval.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="236">
+      <x:c r="A236" t="inlineStr">
+        <x:is>
+          <x:t>CA-PROP64-CA-L06-20261013</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B236" t="inlineStr">
+        <x:is>
+          <x:t>P02-05</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C236" t="inlineStr">
+        <x:is>
+          <x:t>CA</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D236" t="inlineStr">
+        <x:is>
+          <x:t>Both existing Prop64 routes</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E236" t="inlineStr">
+        <x:is>
+          <x:t>Sentence/appeal and actor-owned procedure</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F236" t="inlineStr">
+        <x:is>
+          <x:t>Shared</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G236" t="inlineStr">
+        <x:is>
+          <x:t>BOTH</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H236" t="inlineStr">
+        <x:is>
+          <x:t>Current candidate and existing review report</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I236" t="inlineStr">
+        <x:is>
+          <x:t>NOT RUN</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J236" t="inlineStr">
+        <x:is>
+          <x:t>Qualified decision plus dependent engineering/output/journey acceptance remains active</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K236" t="inlineStr">
+        <x:is>
+          <x:t>docs/rcap/grade-a/handoffs/NATIONWIDE_BLOCKER_RESOLUTION_INPUTS_2026-10-12.md</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L236" t="inlineStr">
+        <x:is>
+          <x:t>Codex engineering; qualified CA reviewer and independent QA</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M236" t="inlineStr">
+        <x:is>
+          <x:t>GA-19 / GA-21 / GA-49</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N236" t="inlineStr">
+        <x:is>
+          <x:t>Precise review matrix; no final disposition or fabricated approval.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:N1"/>

</xml_diff>

<commit_message>
Correct Prop64 form actors and verify source-bound completion duties
</commit_message>
<xml_diff>
--- a/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
+++ b/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
@@ -546,7 +546,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N228" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N239" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Case ID"/>
     <x:tableColumn id="2" name="Control ID"/>
@@ -25207,6 +25207,138 @@
         <x:is>
           <x:t>Precise review matrix; no final disposition or fabricated approval.</x:t>
         </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="237">
+      <x:c r="A237" t="str">
+        <x:v>CA-PROP64-SERVICE-ACTOR-20261013</x:v>
+      </x:c>
+      <x:c r="B237" t="str">
+        <x:v>P04-10</x:v>
+      </x:c>
+      <x:c r="C237" t="str">
+        <x:v>CA</x:v>
+      </x:c>
+      <x:c r="D237" t="str">
+        <x:v>Both existing Prop64 adult routes</x:v>
+      </x:c>
+      <x:c r="E237" t="str">
+        <x:v>CR401 actual nonparty server versus preparer/court</x:v>
+      </x:c>
+      <x:c r="F237" t="str">
+        <x:v>Internal</x:v>
+      </x:c>
+      <x:c r="G237" t="str">
+        <x:v>EN</x:v>
+      </x:c>
+      <x:c r="H237" t="str">
+        <x:v>Current PR268 form-ownership candidate</x:v>
+      </x:c>
+      <x:c r="I237" t="str">
+        <x:v>IN PROGRESS</x:v>
+      </x:c>
+      <x:c r="J237" t="str">
+        <x:v>Source-bound consumer and independent mutations pass. Actual service/signature, legal/language and delivered-journey approval remain pending.</x:v>
+      </x:c>
+      <x:c r="K237" t="str">
+        <x:v>ca-prop64-facts-20261012 / ca-prop64-consumer-independent-20261013</x:v>
+      </x:c>
+      <x:c r="L237" t="str">
+        <x:v>Codex execution; independent agent engineering review</x:v>
+      </x:c>
+      <x:c r="M237" t="str">
+        <x:v>GA-14 / GA-19 / GA-49</x:v>
+      </x:c>
+      <x:c r="N237" t="str">
+        <x:v>Existing official PDF bytes and raster approvals unchanged; no commercial authority.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="238">
+      <x:c r="A238" t="str">
+        <x:v>CA-PROP64-GUIDE-ACTORS-20261013</x:v>
+      </x:c>
+      <x:c r="B238" t="str">
+        <x:v>P05-05</x:v>
+      </x:c>
+      <x:c r="C238" t="str">
+        <x:v>CA</x:v>
+      </x:c>
+      <x:c r="D238" t="str">
+        <x:v>ca-prop64-set CR400/401/403</x:v>
+      </x:c>
+      <x:c r="E238" t="str">
+        <x:v>Caption, optional waivers, actual signing and later service</x:v>
+      </x:c>
+      <x:c r="F238" t="str">
+        <x:v>Internal</x:v>
+      </x:c>
+      <x:c r="G238" t="str">
+        <x:v>EN</x:v>
+      </x:c>
+      <x:c r="H238" t="str">
+        <x:v>Current PR268 form-ownership candidate</x:v>
+      </x:c>
+      <x:c r="I238" t="str">
+        <x:v>IN PROGRESS</x:v>
+      </x:c>
+      <x:c r="J238" t="str">
+        <x:v>Guide now names actual actors and conditional tasks; optional waivers not required; manual signatures retained. Qualified and participant-language review pending.</x:v>
+      </x:c>
+      <x:c r="K238" t="str">
+        <x:v>ca-prop64-facts-20261012 / ca-prop64-consumer-independent-20261013</x:v>
+      </x:c>
+      <x:c r="L238" t="str">
+        <x:v>Codex execution; qualified CA and language reviewers pending</x:v>
+      </x:c>
+      <x:c r="M238" t="str">
+        <x:v>GA-15 / GA-21 / GA-49</x:v>
+      </x:c>
+      <x:c r="N238" t="str">
+        <x:v>Review metadata only; existing approvals do not approve revised text.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="239">
+      <x:c r="A239" t="str">
+        <x:v>CA-PROP64-REMAINING-BINDINGS-20261013</x:v>
+      </x:c>
+      <x:c r="B239" t="str">
+        <x:v>P04-05</x:v>
+      </x:c>
+      <x:c r="C239" t="str">
+        <x:v>CA</x:v>
+      </x:c>
+      <x:c r="D239" t="str">
+        <x:v>ca-prop64-set plus supported juvenile procedure</x:v>
+      </x:c>
+      <x:c r="E239" t="str">
+        <x:v>Known caption/contact/record-section reuse and juvenile binding</x:v>
+      </x:c>
+      <x:c r="F239" t="str">
+        <x:v>Internal</x:v>
+      </x:c>
+      <x:c r="G239" t="str">
+        <x:v>BOTH</x:v>
+      </x:c>
+      <x:c r="H239" t="str">
+        <x:v>Current PR268 form-ownership candidate</x:v>
+      </x:c>
+      <x:c r="I239" t="str">
+        <x:v>FAIL</x:v>
+      </x:c>
+      <x:c r="J239" t="str">
+        <x:v>Actual prepared-input completeness still fails missing required facts and unclassified fields. Bind remaining known facts and source-supported juvenile components, independently verify outputs and journeys.</x:v>
+      </x:c>
+      <x:c r="K239" t="str">
+        <x:v>ca-prop64-facts-20261012 / ca-prop64-consumer-independent-20261013</x:v>
+      </x:c>
+      <x:c r="L239" t="str">
+        <x:v>Codex engineering; independent QA; qualified CA reviewer</x:v>
+      </x:c>
+      <x:c r="M239" t="str">
+        <x:v>GA-14 / GA-15 / GA-19 / GA-21 / GA-43 / GA-49</x:v>
+      </x:c>
+      <x:c r="N239" t="str">
+        <x:v>This checkpoint is not California completion; remaining work stays actively owned.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Bind Prop64 review captions to actual filer and record facts
</commit_message>
<xml_diff>
--- a/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
+++ b/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
@@ -546,7 +546,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N239" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N240" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Case ID"/>
     <x:tableColumn id="2" name="Control ID"/>
@@ -25339,6 +25339,78 @@
       </x:c>
       <x:c r="N239" t="str">
         <x:v>This checkpoint is not California completion; remaining work stays actively owned.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="240">
+      <x:c r="A240" t="inlineStr">
+        <x:is>
+          <x:t>CA-PROP64-CAPTION-CANDIDATE-20261013</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B240" t="inlineStr">
+        <x:is>
+          <x:t>P04-05</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C240" t="inlineStr">
+        <x:is>
+          <x:t>CA</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D240" t="inlineStr">
+        <x:is>
+          <x:t>Both existing Prop64 adult routes</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E240" t="inlineStr">
+        <x:is>
+          <x:t>Self-represented / attorney / long values / conflicting section</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F240" t="inlineStr">
+        <x:is>
+          <x:t>Internal</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G240" t="inlineStr">
+        <x:is>
+          <x:t>EN</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H240" t="inlineStr">
+        <x:is>
+          <x:t>PR268 caption review candidate after401bcf529</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I240" t="inlineStr">
+        <x:is>
+          <x:t>IN PROGRESS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J240" t="inlineStr">
+        <x:is>
+          <x:t>9PDF/12pages:32/32/44 caption writes; no known mapped fact omitted;157root+785independent checks. Actual protected collection, missing facts and qualified approvals remain open.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K240" t="inlineStr">
+        <x:is>
+          <x:t>ca-prop64-facts-20261012/CAPTION-REVIEW-CHECKPOINT-v1.json</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L240" t="inlineStr">
+        <x:is>
+          <x:t>Codex execution; independent engineering/visual review; professional QA pending</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M240" t="inlineStr">
+        <x:is>
+          <x:t>GA-14 / GA-15 / GA-16 / GA-19 / GA-43 / GA-49</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N240" t="inlineStr">
+        <x:is>
+          <x:t>All44 existing artifacts unchanged. Review candidate does not close original production completeness or California.</x:t>
+        </x:is>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Clarify New York sealing guidance by source version and actual actor
</commit_message>
<xml_diff>
--- a/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
+++ b/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
@@ -546,7 +546,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N240" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N241" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Case ID"/>
     <x:tableColumn id="2" name="Control ID"/>
@@ -25410,6 +25410,78 @@
       <x:c r="N240" t="inlineStr">
         <x:is>
           <x:t>All44 existing artifacts unchanged. Review candidate does not close original production completeness or California.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="241">
+      <x:c r="A241" t="inlineStr">
+        <x:is>
+          <x:t>NY-16059-SOURCE-GUIDANCE-20261013</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B241" t="inlineStr">
+        <x:is>
+          <x:t>P04-05</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C241" t="inlineStr">
+        <x:is>
+          <x:t>NY</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D241" t="inlineStr">
+        <x:is>
+          <x:t>NY:discretionary-conviction-sealing-by-petition-under-cpl-160-59</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E241" t="inlineStr">
+        <x:is>
+          <x:t>Current/held execution; 66 conditional flags; actual requester/server</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F241" t="inlineStr">
+        <x:is>
+          <x:t>Internal</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G241" t="inlineStr">
+        <x:is>
+          <x:t>EN</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H241" t="inlineStr">
+        <x:is>
+          <x:t>PR268 guidance candidate after27a0b200a</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I241" t="inlineStr">
+        <x:is>
+          <x:t>IN PROGRESS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J241" t="inlineStr">
+        <x:is>
+          <x:t>194 root + 183 independent checks. 60 non-guide artifacts and 11 neighboring producer outputs unchanged. Typed consumer/current binary/protected delivery/qualified acceptance remain open.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K241" t="inlineStr">
+        <x:is>
+          <x:t>ny-residual-20261012/GUIDANCE-CHECKPOINT-v1.json</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L241" t="inlineStr">
+        <x:is>
+          <x:t>Codex engineering; independent source review; qualified NY/QA pending</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M241" t="inlineStr">
+        <x:is>
+          <x:t>GA-14 / GA-15 / GA-16 / GA-17 / GA-19 / GA-43 / GA-49</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N241" t="inlineStr">
+        <x:is>
+          <x:t>No PDF/approval replacement; no state/finding closure. All 28 expectations retain unexecuted runtime portions.</x:t>
         </x:is>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Use Kansas district facts and preserve financial answer recovery
</commit_message>
<xml_diff>
--- a/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
+++ b/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
@@ -546,7 +546,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N241" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N243" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Case ID"/>
     <x:tableColumn id="2" name="Control ID"/>
@@ -25482,6 +25482,150 @@
       <x:c r="N241" t="inlineStr">
         <x:is>
           <x:t>No PDF/approval replacement; no state/finding closure. All 28 expectations retain unexecuted runtime portions.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="242">
+      <x:c r="A242" t="inlineStr">
+        <x:is>
+          <x:t>KS-DISTRICT-FACTS-20261013</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B242" t="inlineStr">
+        <x:is>
+          <x:t>P03-09</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C242" t="inlineStr">
+        <x:is>
+          <x:t>KS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D242" t="inlineStr">
+        <x:is>
+          <x:t>Existing six candidate paths; district/municipal scope</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E242" t="inlineStr">
+        <x:is>
+          <x:t>Actual election, diversion/specialty/coercion/registration facts</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F242" t="inlineStr">
+        <x:is>
+          <x:t>Public</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G242" t="inlineStr">
+        <x:is>
+          <x:t>BOTH</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H242" t="inlineStr">
+        <x:is>
+          <x:t>PR268 after bcb1e69f0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I242" t="inlineStr">
+        <x:is>
+          <x:t>IN PROGRESS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J242" t="inlineStr">
+        <x:is>
+          <x:t>1671 root and3386 independent checks; two actual anonymous browser flows. Statutory predicates, protected delivery and qualified acceptance remain open.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K242" t="inlineStr">
+        <x:is>
+          <x:t>ks-district-facts-20261013/CHECKPOINT-v1.json</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L242" t="inlineStr">
+        <x:is>
+          <x:t>Codex engineering; independent source/QA; qualified KS reviewer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M242" t="inlineStr">
+        <x:is>
+          <x:t>GA-10 / GA-12 / GA-17 / GA-21 / GA-43</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N242" t="inlineStr">
+        <x:is>
+          <x:t>All28 source obligations retained; held results are not final supported-route dispositions.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="243">
+      <x:c r="A243" t="inlineStr">
+        <x:is>
+          <x:t>FINANCIAL-UNKNOWN-RECOVERY-20261013</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B243" t="inlineStr">
+        <x:is>
+          <x:t>P04-05</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C243" t="inlineStr">
+        <x:is>
+          <x:t>MS / shared exact contracts</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D243" t="inlineStr">
+        <x:is>
+          <x:t>Existing financial carry and independent-paid contracts</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E243" t="inlineStr">
+        <x:is>
+          <x:t>Raw incompatible value, old positive result, explicit correction</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F243" t="inlineStr">
+        <x:is>
+          <x:t>Internal</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G243" t="inlineStr">
+        <x:is>
+          <x:t>BOTH</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H243" t="inlineStr">
+        <x:is>
+          <x:t>PR268 after bcb1e69f0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I243" t="inlineStr">
+        <x:is>
+          <x:t>IN PROGRESS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J243" t="inlineStr">
+        <x:is>
+          <x:t>139 exact paid facts visible; genuine old malformed-payment defect corrected. Actual local EN21/ES22 owner browser/API/DB checks; raw history and cleanup proved.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K243" t="inlineStr">
+        <x:is>
+          <x:t>ks-district-facts-20261013/CHECKPOINT-v1.json</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L243" t="inlineStr">
+        <x:is>
+          <x:t>Codex engineering; independent review; professional QA pending</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M243" t="inlineStr">
+        <x:is>
+          <x:t>GA-10 / GA-43</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N243" t="inlineStr">
+        <x:is>
+          <x:t>Non-plan correction residual outside carry contracts stays actively owned; no payment or release acceptance.</x:t>
         </x:is>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Preserve held financial corrections through screening and saved matters
</commit_message>
<xml_diff>
--- a/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
+++ b/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
@@ -546,7 +546,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N243" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N244" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Case ID"/>
     <x:tableColumn id="2" name="Control ID"/>
@@ -25626,6 +25626,78 @@
       <x:c r="N243" t="inlineStr">
         <x:is>
           <x:t>Non-plan correction residual outside carry contracts stays actively owned; no payment or release acceptance.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="244">
+      <x:c r="A244" t="inlineStr">
+        <x:is>
+          <x:t>FINANCIAL-NOPLAN-CORRECTION-20261013</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B244" t="inlineStr">
+        <x:is>
+          <x:t>P04-05</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C244" t="inlineStr">
+        <x:is>
+          <x:t>LA/MO/NC/NE/VT/WV + shared status controls</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D244" t="inlineStr">
+        <x:is>
+          <x:t>13 existing positive witnesses; exact139 paid contracts</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E244" t="inlineStr">
+        <x:is>
+          <x:t>Held no-plan correction, raw preservation, visible questions, autosave</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F244" t="inlineStr">
+        <x:is>
+          <x:t>Internal</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G244" t="inlineStr">
+        <x:is>
+          <x:t>BOTH</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H244" t="inlineStr">
+        <x:is>
+          <x:t>PR268 after01d6888a9</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I244" t="inlineStr">
+        <x:is>
+          <x:t>IN PROGRESS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J244" t="inlineStr">
+        <x:is>
+          <x:t>1359 focused checks; local EN34/ES35 protected owner checks; four EN/ES screening flows; actual RCAP admission/autosave16 checks. No authority invented.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K244" t="inlineStr">
+        <x:is>
+          <x:t>ks-district-facts-20261013/NONPLAN-CHECKPOINT-v1.json</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L244" t="inlineStr">
+        <x:is>
+          <x:t>Codex engineering; independent engineering review; qualified QA/language pending</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M244" t="inlineStr">
+        <x:is>
+          <x:t>GA-10 / GA-43</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N244" t="inlineStr">
+        <x:is>
+          <x:t>Historical malformed null-route records, DE profile schema and residual EN/ES labels remain actively owned; no finding or state closure.</x:t>
         </x:is>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Restore Delaware date controls in the strict public profile
</commit_message>
<xml_diff>
--- a/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
+++ b/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
@@ -546,7 +546,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N244" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N245" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Case ID"/>
     <x:tableColumn id="2" name="Control ID"/>
@@ -25698,6 +25698,78 @@
       <x:c r="N244" t="inlineStr">
         <x:is>
           <x:t>Historical malformed null-route records, DE profile schema and residual EN/ES labels remain actively owned; no finding or state closure.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="245">
+      <x:c r="A245" t="inlineStr">
+        <x:is>
+          <x:t>DE-PUBLIC-DATE-SCHEMA-20261013</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B245" t="inlineStr">
+        <x:is>
+          <x:t>P03-09</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C245" t="inlineStr">
+        <x:is>
+          <x:t>DE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D245" t="inlineStr">
+        <x:is>
+          <x:t>Existing adult-conviction screening</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E245" t="inlineStr">
+        <x:is>
+          <x:t>Four conditional date controls; known/unknown values</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F245" t="inlineStr">
+        <x:is>
+          <x:t>Public</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G245" t="inlineStr">
+        <x:is>
+          <x:t>BOTH</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H245" t="inlineStr">
+        <x:is>
+          <x:t>PR268 after46116aa19</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I245" t="inlineStr">
+        <x:is>
+          <x:t>IN PROGRESS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J245" t="inlineStr">
+        <x:is>
+          <x:t>Actual HTTP profile and strict frontend schema now load;30 root checks,16 real browser input cases, existing2687 predicate checks preserved.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K245" t="inlineStr">
+        <x:is>
+          <x:t>de-timing-exclusions-20261012/PROFILE-DATES-CHECKPOINT-v1.json</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L245" t="inlineStr">
+        <x:is>
+          <x:t>Codex engineering; independent source/runtime review; qualified acceptance pending</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M245" t="inlineStr">
+        <x:is>
+          <x:t>GA-20 / GA-43</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N245" t="inlineStr">
+        <x:is>
+          <x:t>Four options:null descriptor additions only. Remaining97 downstream appearances and source/documents/journeys remain owned.</x:t>
         </x:is>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Preserve factual exclusions and saved IL GA owner recovery
</commit_message>
<xml_diff>
--- a/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
+++ b/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
@@ -546,7 +546,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N245" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N246" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Case ID"/>
     <x:tableColumn id="2" name="Control ID"/>
@@ -25770,6 +25770,78 @@
       <x:c r="N245" t="inlineStr">
         <x:is>
           <x:t>Four options:null descriptor additions only. Remaining97 downstream appearances and source/documents/journeys remain owned.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="246">
+      <x:c r="A246" t="inlineStr">
+        <x:is>
+          <x:t>IL-GA-FACTUAL-EXCLUSION-RECOVERY-20261013</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B246" t="inlineStr">
+        <x:is>
+          <x:t>P03-09</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C246" t="inlineStr">
+        <x:is>
+          <x:t>IL / GA</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D246" t="inlineStr">
+        <x:is>
+          <x:t>Cannabis and original First Offender exclusions</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E246" t="inlineStr">
+        <x:is>
+          <x:t>Exact negative facts; historical protected ownership and explicit correction</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F246" t="inlineStr">
+        <x:is>
+          <x:t>Public / owner Briefcase</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G246" t="inlineStr">
+        <x:is>
+          <x:t>BOTH</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H246" t="inlineStr">
+        <x:is>
+          <x:t>PR268 afterbd4f9715b</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I246" t="inlineStr">
+        <x:is>
+          <x:t>IN PROGRESS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J246" t="inlineStr">
+        <x:is>
+          <x:t>Contradicted optional hints no longer select excluded procedures. Genuine old held rows remain readable without current packet authority; explicit owner corrections and conditional continuation pass local browser/DB/CAS.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K246" t="inlineStr">
+        <x:is>
+          <x:t>ga21-independent-residual-20261013/IL-GA-CHECKPOINT-v1.json</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L246" t="inlineStr">
+        <x:is>
+          <x:t>Codex engineering; independent evidence review; qualified acceptance pending</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M246" t="inlineStr">
+        <x:is>
+          <x:t>GA-21 / GA-43</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N246" t="inlineStr">
+        <x:is>
+          <x:t>Truthful alternative requests, empty-hint conviction/nonconviction fallback, MS date reachability and all original16 findings remain actively owned; no route/financial/release approval.</x:t>
         </x:is>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Restore exact Mississippi timing inputs and safe saved-date recovery
</commit_message>
<xml_diff>
--- a/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
+++ b/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
@@ -546,7 +546,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N246" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N247" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Case ID"/>
     <x:tableColumn id="2" name="Control ID"/>
@@ -25842,6 +25842,78 @@
       <x:c r="N246" t="inlineStr">
         <x:is>
           <x:t>Truthful alternative requests, empty-hint conviction/nonconviction fallback, MS date reachability and all original16 findings remain actively owned; no route/financial/release approval.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="247">
+      <x:c r="A247" t="inlineStr">
+        <x:is>
+          <x:t>MS-EXACT-TIMING-RECOVERY-20261013</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B247" t="inlineStr">
+        <x:is>
+          <x:t>P03-09</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C247" t="inlineStr">
+        <x:is>
+          <x:t>MS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D247" t="inlineStr">
+        <x:is>
+          <x:t>Six existing timing facts and calendar recovery</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E247" t="inlineStr">
+        <x:is>
+          <x:t>Source-required controls; exact dates; saved and verified record correction</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F247" t="inlineStr">
+        <x:is>
+          <x:t>Public / owner Briefcase / RCAP draft</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G247" t="inlineStr">
+        <x:is>
+          <x:t>BOTH</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H247" t="inlineStr">
+        <x:is>
+          <x:t>PR268 after8fcb4f7b</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I247" t="inlineStr">
+        <x:is>
+          <x:t>IN PROGRESS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J247" t="inlineStr">
+        <x:is>
+          <x:t>Six existing controls reachable; invalid calendar dates hold; historical unverified and genuinely old-engine verified records readable/correctable with no inherited readiness. Deadline crossing uses isolated historical full-tuple proof.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K247" t="inlineStr">
+        <x:is>
+          <x:t>ms-exact-timing-20261013/MS-TIMING-CHECKPOINT-v1.json</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L247" t="inlineStr">
+        <x:is>
+          <x:t>Codex engineering; independent evidence review; qualified acceptance pending</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M247" t="inlineStr">
+        <x:is>
+          <x:t>GA-21 / GA-43</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N247" t="inlineStr">
+        <x:is>
+          <x:t>Current-primary/language review, real hosted/offered journeys, MS residual routing and all original16 remain actively owned; no financial/release approval.</x:t>
         </x:is>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Preserve exact New York completion conditions through packet review
</commit_message>
<xml_diff>
--- a/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
+++ b/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
@@ -546,7 +546,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N247" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N248" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Case ID"/>
     <x:tableColumn id="2" name="Control ID"/>
@@ -25914,6 +25914,78 @@
       <x:c r="N247" t="inlineStr">
         <x:is>
           <x:t>Current-primary/language review, real hosted/offered journeys, MS residual routing and all original16 remain actively owned; no financial/release approval.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="248">
+      <x:c r="A248" t="inlineStr">
+        <x:is>
+          <x:t>NY-TYPED-COMPLETION-20261013</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B248" t="inlineStr">
+        <x:is>
+          <x:t>P03-09</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C248" t="inlineStr">
+        <x:is>
+          <x:t>NY</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D248" t="inlineStr">
+        <x:is>
+          <x:t>Exact source conditions and completion actors</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E248" t="inlineStr">
+        <x:is>
+          <x:t>68 retained form obligations; preserve known facts and all fields</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F248" t="inlineStr">
+        <x:is>
+          <x:t>Held CPL160.59 review family</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G248" t="inlineStr">
+        <x:is>
+          <x:t>EN source instructions</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H248" t="inlineStr">
+        <x:is>
+          <x:t>PR268 afterb7955164c</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I248" t="inlineStr">
+        <x:is>
+          <x:t>IN PROGRESS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J248" t="inlineStr">
+        <x:is>
+          <x:t>66 blanket-required rows and two actor errors corrected with typed declarations. Reader rejects absent source, forged proof and untrusted applicability; actual audit retains68 unresolved blanks.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K248" t="inlineStr">
+        <x:is>
+          <x:t>ny-residual-20261012/NY-TYPED-CHECKPOINT-v1.json</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L248" t="inlineStr">
+        <x:is>
+          <x:t>Codex engineering; independent review; qualified acceptance pending</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M248" t="inlineStr">
+        <x:is>
+          <x:t>GA-49</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N248" t="inlineStr">
+        <x:is>
+          <x:t>Original and current source custody, trusted protected facts, positive source-bound tests, current form renderer/delivery and legal/language/QA approvals remain owned.</x:t>
         </x:is>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Collect and preserve exact California court caption facts
</commit_message>
<xml_diff>
--- a/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
+++ b/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
@@ -546,7 +546,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N248" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N249" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Case ID"/>
     <x:tableColumn id="2" name="Control ID"/>
@@ -25986,6 +25986,78 @@
       <x:c r="N248" t="inlineStr">
         <x:is>
           <x:t>Original and current source custody, trusted protected facts, positive source-bound tests, current form renderer/delivery and legal/language/QA approvals remain owned.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="249">
+      <x:c r="A249" t="inlineStr">
+        <x:is>
+          <x:t>CA-PROTECTED-CAPTION-20261013</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B249" t="inlineStr">
+        <x:is>
+          <x:t>P03-09</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C249" t="inlineStr">
+        <x:is>
+          <x:t>CA</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D249" t="inlineStr">
+        <x:is>
+          <x:t>Protected caption collection and source rendering</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E249" t="inlineStr">
+        <x:is>
+          <x:t>Defendant name, exact court case, filing county and actual filer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F249" t="inlineStr">
+        <x:is>
+          <x:t>Ordinary owner ENES / official adult review PDFs</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G249" t="inlineStr">
+        <x:is>
+          <x:t>BOTH</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H249" t="inlineStr">
+        <x:is>
+          <x:t>PR268 afterf898a765f</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I249" t="inlineStr">
+        <x:is>
+          <x:t>IN PROGRESS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J249" t="inlineStr">
+        <x:is>
+          <x:t>Four packet-only facts; strict prior/current source context; actual owner saves bind official source captions. Prior verification is held until required facts are supplied and explicitly reviewed.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K249" t="inlineStr">
+        <x:is>
+          <x:t>ca-prop64-facts-20261012/CAPTION-COLLECTION-CHECKPOINT-v1.json</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L249" t="inlineStr">
+        <x:is>
+          <x:t>Codex engineering; independent evidence review; qualified acceptance pending</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M249" t="inlineStr">
+        <x:is>
+          <x:t>GA-49 / GA-43</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N249" t="inlineStr">
+        <x:is>
+          <x:t>Remaining30contact/address obligations, service/judicial/signature completion, juvenile/current-source/qualified acceptance and authorized fulfillment/delivery remain active.</x:t>
         </x:is>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Collect requested conviction relief and preserve protected corrections
</commit_message>
<xml_diff>
--- a/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
+++ b/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
@@ -546,7 +546,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N249" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N250" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Case ID"/>
     <x:tableColumn id="2" name="Control ID"/>
@@ -26058,6 +26058,78 @@
       <x:c r="N249" t="inlineStr">
         <x:is>
           <x:t>Remaining30contact/address obligations, service/judicial/signature completion, juvenile/current-source/qualified acceptance and authorized fulfillment/delivery remain active.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="250">
+      <x:c r="A250" t="inlineStr">
+        <x:is>
+          <x:t>CONVICTION-REQUEST-20261013</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B250" t="inlineStr">
+        <x:is>
+          <x:t>P03-09</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C250" t="inlineStr">
+        <x:is>
+          <x:t>MS / GA / IL</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D250" t="inlineStr">
+        <x:is>
+          <x:t>Actual requested relief and conviction-safe fallback</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E250" t="inlineStr">
+        <x:is>
+          <x:t>No optional hint or compiled singleton establishes a nonconviction</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F250" t="inlineStr">
+        <x:is>
+          <x:t>Public ENES and authenticated protected correction</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G250" t="inlineStr">
+        <x:is>
+          <x:t>BOTH</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H250" t="inlineStr">
+        <x:is>
+          <x:t>PR268 after706dfe818</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I250" t="inlineStr">
+        <x:is>
+          <x:t>IN PROGRESS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J250" t="inlineStr">
+        <x:is>
+          <x:t>Ten explicit request/fact questions preserve original facts and select only supported candidates; 81 genuine predecessors remain readable and correctable without inherited readiness.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K250" t="inlineStr">
+        <x:is>
+          <x:t>ga21-independent-residual-20261013/FALLBACK-CHECKPOINT-v1.json</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L250" t="inlineStr">
+        <x:is>
+          <x:t>Codex engineering; independent review; qualified decision pending</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M250" t="inlineStr">
+        <x:is>
+          <x:t>GA-21 / GA-43</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N250" t="inlineStr">
+        <x:is>
+          <x:t>Program/mixed/later event predicates, all source eligibility/authority, legal/bilingual acceptance and all 16 findings remain actively owned.</x:t>
         </x:is>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Collect owned NY sealing packet facts with protected provenance
</commit_message>
<xml_diff>
--- a/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
+++ b/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
@@ -546,7 +546,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N250" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N251" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Case ID"/>
     <x:tableColumn id="2" name="Control ID"/>
@@ -26130,6 +26130,78 @@
       <x:c r="N250" t="inlineStr">
         <x:is>
           <x:t>Program/mixed/later event predicates, all source eligibility/authority, legal/bilingual acceptance and all 16 findings remain actively owned.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="251">
+      <x:c r="A251" t="inlineStr">
+        <x:is>
+          <x:t>NY-PACKET-PREPARATION-20261013</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B251" t="inlineStr">
+        <x:is>
+          <x:t>P03-09 / P04</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C251" t="inlineStr">
+        <x:is>
+          <x:t>NY</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D251" t="inlineStr">
+        <x:is>
+          <x:t>CPL160.59 owned packet facts and current logical components</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E251" t="inlineStr">
+        <x:is>
+          <x:t>Exact owner facts do not establish source custody or later acts</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F251" t="inlineStr">
+        <x:is>
+          <x:t>Packet Information ENES and authenticated preparation projection</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G251" t="inlineStr">
+        <x:is>
+          <x:t>BOTH</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H251" t="inlineStr">
+        <x:is>
+          <x:t>PR268 after fafc82a40</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I251" t="inlineStr">
+        <x:is>
+          <x:t>IN PROGRESS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J251" t="inlineStr">
+        <x:is>
+          <x:t>Ten packet-only controls preserve actual identifiers, raw maps and semantic history; four narrow conditions derive only from valid owned answers.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K251" t="inlineStr">
+        <x:is>
+          <x:t>ny-residual-20261012/PACKET-PREPARATION-CHECKPOINT-v1.json</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L251" t="inlineStr">
+        <x:is>
+          <x:t>Codex engineering; independent review; qualified decisions pending</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M251" t="inlineStr">
+        <x:is>
+          <x:t>GA-49 / GA-43</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N251" t="inlineStr">
+        <x:is>
+          <x:t>Source bytes, 68-row consumer acceptance, remaining court/case/statement/attachment requirements, qualified reviews and delivery remain active.</x:t>
         </x:is>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Connect owned NY facts to source-bound completeness diagnostics
</commit_message>
<xml_diff>
--- a/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
+++ b/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
@@ -546,7 +546,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N251" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N252" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Case ID"/>
     <x:tableColumn id="2" name="Control ID"/>
@@ -26202,6 +26202,78 @@
       <x:c r="N251" t="inlineStr">
         <x:is>
           <x:t>Source bytes, 68-row consumer acceptance, remaining court/case/statement/attachment requirements, qualified reviews and delivery remain active.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="252">
+      <x:c r="A252" t="inlineStr">
+        <x:is>
+          <x:t>NY-OWNED-CONSUMER-20261013</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B252" t="inlineStr">
+        <x:is>
+          <x:t>P03-09 / P04</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C252" t="inlineStr">
+        <x:is>
+          <x:t>NY</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D252" t="inlineStr">
+        <x:is>
+          <x:t>Authenticated owner facts in typed completeness consumer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E252" t="inlineStr">
+        <x:is>
+          <x:t>Serialized flags and fixture PDFs confer no owner/source authority</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F252" t="inlineStr">
+        <x:is>
+          <x:t>Owned read, ENES, exact68-row diagnostics</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G252" t="inlineStr">
+        <x:is>
+          <x:t>BOTH</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H252" t="inlineStr">
+        <x:is>
+          <x:t>PR268 after7838f1e91</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I252" t="inlineStr">
+        <x:is>
+          <x:t>IN PROGRESS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J252" t="inlineStr">
+        <x:is>
+          <x:t>Private server resolver after existing owner read;17 narrow applicability rows and5 known-value gaps,51 untouched.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K252" t="inlineStr">
+        <x:is>
+          <x:t>ny-residual-20261012/OWNED-CONSUMER-CHECKPOINT-v1.json</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L252" t="inlineStr">
+        <x:is>
+          <x:t>Codex engineering; independent review; source/qualified pending</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M252" t="inlineStr">
+        <x:is>
+          <x:t>GA-49 / GA-43</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N252" t="inlineStr">
+        <x:is>
+          <x:t>Authentic source positive acceptance, actual per-case associations, court/statement/attachments, approvals and protected delivery remain active.</x:t>
         </x:is>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Collect and preserve New York case records with owned coherence checks
</commit_message>
<xml_diff>
--- a/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
+++ b/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
@@ -546,7 +546,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N252" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N253" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Case ID"/>
     <x:tableColumn id="2" name="Control ID"/>
@@ -26274,6 +26274,78 @@
       <x:c r="N252" t="inlineStr">
         <x:is>
           <x:t>Authentic source positive acceptance, actual per-case associations, court/statement/attachments, approvals and protected delivery remain active.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="253">
+      <x:c r="A253" t="inlineStr">
+        <x:is>
+          <x:t>NY-CASE-COLLECTION-20261013</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B253" t="inlineStr">
+        <x:is>
+          <x:t>P03-09 / P04</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C253" t="inlineStr">
+        <x:is>
+          <x:t>NY</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D253" t="inlineStr">
+        <x:is>
+          <x:t>Actual per-case records, filing destination and applicant statement</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E253" t="inlineStr">
+        <x:is>
+          <x:t>No flattening, automatic grouping, or inherited verification</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F253" t="inlineStr">
+        <x:is>
+          <x:t>Old verified recovery, ENES save/review/history/CAS, per-case clock conflicts</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G253" t="inlineStr">
+        <x:is>
+          <x:t>BOTH</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H253" t="inlineStr">
+        <x:is>
+          <x:t>PR268 afterf330ca64a</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I253" t="inlineStr">
+        <x:is>
+          <x:t>IN PROGRESS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J253" t="inlineStr">
+        <x:is>
+          <x:t>Six packet-only controls; stable case/offense/sentence/release identity, exact inventory confirmation and readable recovery.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K253" t="inlineStr">
+        <x:is>
+          <x:t>ny-residual-20261012/CASE-COLLECTION-CHECKPOINT-v1.json</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L253" t="inlineStr">
+        <x:is>
+          <x:t>Codex engineering; independent review; qualified source/language pending</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M253" t="inlineStr">
+        <x:is>
+          <x:t>GA-49 / GA-43 / GA-19</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N253" t="inlineStr">
+        <x:is>
+          <x:t>Source-bound class/statute/count/venue/prosecutor/attachment interpretation, exact sources/output, approval and protected delivery remain actively owned.</x:t>
         </x:is>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Localize protected generated matter titles with exact route copy
</commit_message>
<xml_diff>
--- a/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
+++ b/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
@@ -546,7 +546,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N253" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N254" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Case ID"/>
     <x:tableColumn id="2" name="Control ID"/>
@@ -26346,6 +26346,78 @@
       <x:c r="N253" t="inlineStr">
         <x:is>
           <x:t>Source-bound class/statute/count/venue/prosecutor/attachment interpretation, exact sources/output, approval and protected delivery remain actively owned.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="254">
+      <x:c r="A254" t="inlineStr">
+        <x:is>
+          <x:t>GA43-TITLES-20261013</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B254" t="inlineStr">
+        <x:is>
+          <x:t>P03/P10</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C254" t="inlineStr">
+        <x:is>
+          <x:t>Nationwide reviewed route labels</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D254" t="inlineStr">
+        <x:is>
+          <x:t>Generated protected matter titles in EN/ES</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E254" t="inlineStr">
+        <x:is>
+          <x:t>Reuse exact route+original copy; preserve other titles</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F254" t="inlineStr">
+        <x:is>
+          <x:t>350 route pairs plus actual ordinary-owner pages</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G254" t="inlineStr">
+        <x:is>
+          <x:t>BOTH</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H254" t="inlineStr">
+        <x:is>
+          <x:t>PR268 after2a27c1cde</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I254" t="inlineStr">
+        <x:is>
+          <x:t>IN PROGRESS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J254" t="inlineStr">
+        <x:is>
+          <x:t>Seven direct title slots use existing bilingual metadata without changing authority or saved records.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K254" t="inlineStr">
+        <x:is>
+          <x:t>ga43-generated-titles-20261013/TITLE-CHECKPOINT-v1.json</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L254" t="inlineStr">
+        <x:is>
+          <x:t>Codex engineering / independent review</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M254" t="inlineStr">
+        <x:is>
+          <x:t>GA-43</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N254" t="inlineStr">
+        <x:is>
+          <x:t>Dynamic title sentences, subtitles, summaries, components, categories and full journey/language/device approval remain actively owned.</x:t>
         </x:is>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Preserve record-bound NY classifications and adverse-result case correction
</commit_message>
<xml_diff>
--- a/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
+++ b/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
@@ -546,7 +546,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N254" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N255" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Case ID"/>
     <x:tableColumn id="2" name="Control ID"/>
@@ -26418,6 +26418,78 @@
       <x:c r="N254" t="inlineStr">
         <x:is>
           <x:t>Dynamic title sentences, subtitles, summaries, components, categories and full journey/language/device approval remain actively owned.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="255">
+      <x:c r="A255" t="inlineStr">
+        <x:is>
+          <x:t>NY-CASE-CLASSIFICATION-20261013</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B255" t="inlineStr">
+        <x:is>
+          <x:t>P02 / P03-09 / P04</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C255" t="inlineStr">
+        <x:is>
+          <x:t>NY</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D255" t="inlineStr">
+        <x:is>
+          <x:t>Record-bound conviction classification and contradiction correction</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E255" t="inlineStr">
+        <x:is>
+          <x:t>No inferred class, exclusions, legal grouping or inherited verification</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F255" t="inlineStr">
+        <x:is>
+          <x:t>Legacy recovery; per-answer staleness; ENES saved/reviewed owner journey</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G255" t="inlineStr">
+        <x:is>
+          <x:t>BOTH</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H255" t="inlineStr">
+        <x:is>
+          <x:t>PR268 after97d6f01</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I255" t="inlineStr">
+        <x:is>
+          <x:t>IN PROGRESS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J255" t="inlineStr">
+        <x:is>
+          <x:t>Explicit record classes and eight source categories; normalized conflicts and independent answer reconfirmation.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K255" t="inlineStr">
+        <x:is>
+          <x:t>ny-residual-20261012/CLASSIFICATION-CHECKPOINT-v1.json</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L255" t="inlineStr">
+        <x:is>
+          <x:t>Codex engineering; independent review; qualified legal/language pending</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M255" t="inlineStr">
+        <x:is>
+          <x:t>GA-19 / GA-43 / GA-49</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N255" t="inlineStr">
+        <x:is>
+          <x:t>Actual statute/version/subdivision/history/grouping, venue/prosecutor/attachments, authentic sources/output, approvals and delivery remain actively owned.</x:t>
         </x:is>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
test: restore protected presentation boundary execution
</commit_message>
<xml_diff>
--- a/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
+++ b/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
@@ -546,7 +546,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N255" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N256" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Case ID"/>
     <x:tableColumn id="2" name="Control ID"/>
@@ -26490,6 +26490,78 @@
       <x:c r="N255" t="inlineStr">
         <x:is>
           <x:t>Actual statute/version/subdivision/history/grouping, venue/prosecutor/attachments, authentic sources/output, approvals and delivery remain actively owned.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="256">
+      <x:c r="A256" t="inlineStr">
+        <x:is>
+          <x:t>GA43-PRESENTATION-HARNESS-20261013</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B256" t="inlineStr">
+        <x:is>
+          <x:t>P09 / P11</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C256" t="inlineStr">
+        <x:is>
+          <x:t>ALL</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D256" t="inlineStr">
+        <x:is>
+          <x:t>Restore protected presentation boundary regression execution</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E256" t="inlineStr">
+        <x:is>
+          <x:t>All original assertions retained; no runtime behavior or authority change</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F256" t="inlineStr">
+        <x:is>
+          <x:t>Original102 assertion sites plus5 no-plan cases and actual disposable PostgreSQL</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G256" t="inlineStr">
+        <x:is>
+          <x:t>BOTH</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H256" t="inlineStr">
+        <x:is>
+          <x:t>PR268 after253389316</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I256" t="inlineStr">
+        <x:is>
+          <x:t>IN PROGRESS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J256" t="inlineStr">
+        <x:is>
+          <x:t>Real source imports replace missing aliases; fixture forwards its actual protected plan.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K256" t="inlineStr">
+        <x:is>
+          <x:t>ga43-generated-titles-20261013/HARNESS-CHECKPOINT-v1.json</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L256" t="inlineStr">
+        <x:is>
+          <x:t>Codex engineering; independent bounded review</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M256" t="inlineStr">
+        <x:is>
+          <x:t>GA-43 / GA-44</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N256" t="inlineStr">
+        <x:is>
+          <x:t>Remaining presentation copy, all route journeys, hosted/schema/worker acceptance and external approvals stay actively owned.</x:t>
         </x:is>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
feat: collect protected California filer and court contacts
</commit_message>
<xml_diff>
--- a/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
+++ b/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
@@ -546,7 +546,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N256" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N257" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Case ID"/>
     <x:tableColumn id="2" name="Control ID"/>
@@ -26562,6 +26562,78 @@
       <x:c r="N256" t="inlineStr">
         <x:is>
           <x:t>Remaining presentation copy, all route journeys, hosted/schema/worker acceptance and external approvals stay actively owned.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="257">
+      <x:c r="A257" t="inlineStr">
+        <x:is>
+          <x:t>CA-PROTECTED-CONTACT-20261013</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B257" t="inlineStr">
+        <x:is>
+          <x:t>P03 / P04 / P09 / P10</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C257" t="inlineStr">
+        <x:is>
+          <x:t>CA</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D257" t="inlineStr">
+        <x:is>
+          <x:t>Filer and court contacts reach protected source captions</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E257" t="inlineStr">
+        <x:is>
+          <x:t>Bound actor/court details, explicit optional states, old records preserved</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F257" t="inlineStr">
+        <x:is>
+          <x:t>Two adult routes x two filer actors x ENES;12 source PDFs16pages</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G257" t="inlineStr">
+        <x:is>
+          <x:t>BOTH</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H257" t="inlineStr">
+        <x:is>
+          <x:t>PR268 aftera4430f3cc</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I257" t="inlineStr">
+        <x:is>
+          <x:t>IN PROGRESS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J257" t="inlineStr">
+        <x:is>
+          <x:t>Strict structured records; stale identity binding; optional facts retained; protected save/review and exact historical successor.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K257" t="inlineStr">
+        <x:is>
+          <x:t>ca-prop64-facts-20261012/CONTACT-CHECKPOINT-v1.json</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L257" t="inlineStr">
+        <x:is>
+          <x:t>Codex engineering; independent review; qualified decisions pending</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M257" t="inlineStr">
+        <x:is>
+          <x:t>GA-15 / GA-16 / GA-19 / GA-43 / GA-49</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N257" t="inlineStr">
+        <x:is>
+          <x:t>Contact exceptions/copy approval, adult/juvenile/source decisions, service/signature/judicial duties, full/court-only assembly, authorized fulfillment/delivery and all16 stay active.</x:t>
         </x:is>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Reconcile New York filing courts with record-bound offense classes
</commit_message>
<xml_diff>
--- a/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
+++ b/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
@@ -546,7 +546,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N257" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N258" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Case ID"/>
     <x:tableColumn id="2" name="Control ID"/>
@@ -26634,6 +26634,78 @@
       <x:c r="N257" t="inlineStr">
         <x:is>
           <x:t>Contact exceptions/copy approval, adult/juvenile/source decisions, service/signature/judicial duties, full/court-only assembly, authorized fulfillment/delivery and all16 stay active.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="258">
+      <x:c r="A258" t="inlineStr">
+        <x:is>
+          <x:t>NY-FILING-VENUE-20261013</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B258" t="inlineStr">
+        <x:is>
+          <x:t>P02 / P03-09 / P04</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C258" t="inlineStr">
+        <x:is>
+          <x:t>NY</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D258" t="inlineStr">
+        <x:is>
+          <x:t>Record-bound class and filing-court reconciliation</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E258" t="inlineStr">
+        <x:is>
+          <x:t>No inferred grade, court transfer, grouping or legal approval</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F258" t="inlineStr">
+        <x:is>
+          <x:t>Genuine saved verification recovery; actual ENES owner persistence and conflict recovery</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G258" t="inlineStr">
+        <x:is>
+          <x:t>BOTH</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H258" t="inlineStr">
+        <x:is>
+          <x:t>PR268 after20b2f0adc</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I258" t="inlineStr">
+        <x:is>
+          <x:t>IN PROGRESS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J258" t="inlineStr">
+        <x:is>
+          <x:t>Explicit exact classes where competing courts require them; known venue contradictions; retained direction review facts.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K258" t="inlineStr">
+        <x:is>
+          <x:t>ny-residual-20261012/VENUE-CHECKPOINT-v1.json</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L258" t="inlineStr">
+        <x:is>
+          <x:t>Codex engineering; independent review; qualified legal/language pending</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M258" t="inlineStr">
+        <x:is>
+          <x:t>GA-16 / GA-19 / GA-43 / GA-49</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N258" t="inlineStr">
+        <x:is>
+          <x:t>Complete-history/prior orders/incarceration/grouping, authentic sources/output, qualified approval and delivery remain actively owned.</x:t>
         </x:is>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Preserve New York prior applications and entered sealing orders
</commit_message>
<xml_diff>
--- a/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
+++ b/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
@@ -546,7 +546,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N258" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N259" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Case ID"/>
     <x:tableColumn id="2" name="Control ID"/>
@@ -26706,6 +26706,78 @@
       <x:c r="N258" t="inlineStr">
         <x:is>
           <x:t>Complete-history/prior orders/incarceration/grouping, authentic sources/output, qualified approval and delivery remain actively owned.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="259">
+      <x:c r="A259" t="inlineStr">
+        <x:is>
+          <x:t>NY-PRIOR-APPLICATIONS-20261013</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B259" t="inlineStr">
+        <x:is>
+          <x:t>P02 / P03-09 / P04</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C259" t="inlineStr">
+        <x:is>
+          <x:t>NY</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D259" t="inlineStr">
+        <x:is>
+          <x:t>Earlier applications and actual entered sealing orders</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E259" t="inlineStr">
+        <x:is>
+          <x:t>Court own motion is not participant application; no inferred maximum</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F259" t="inlineStr">
+        <x:is>
+          <x:t>Exact old verified successors, held editor and ENES ordinary persistence</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G259" t="inlineStr">
+        <x:is>
+          <x:t>BOTH</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H259" t="inlineStr">
+        <x:is>
+          <x:t>PR268 after826036ad9</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I259" t="inlineStr">
+        <x:is>
+          <x:t>IN PROGRESS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J259" t="inlineStr">
+        <x:is>
+          <x:t>Separate application outcomes, actual orders/components and later unsealing; original facts reused with provenance.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K259" t="inlineStr">
+        <x:is>
+          <x:t>ny-residual-20261012/HISTORY-CHECKPOINT-v1.json</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L259" t="inlineStr">
+        <x:is>
+          <x:t>Codex engineering; independent reviewer; qualified decisions pending</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M259" t="inlineStr">
+        <x:is>
+          <x:t>GA-17 / GA-19 / GA-43 / GA-49</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N259" t="inlineStr">
+        <x:is>
+          <x:t>Future-law/repeating intents, complete history/grouping/clock, source/copies/output/legal/language/fulfillment remain owned.</x:t>
         </x:is>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Preserve New York intended future sealing applications
</commit_message>
<xml_diff>
--- a/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
+++ b/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
@@ -546,7 +546,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N259" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N260" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Case ID"/>
     <x:tableColumn id="2" name="Control ID"/>
@@ -26778,6 +26778,78 @@
       <x:c r="N259" t="inlineStr">
         <x:is>
           <x:t>Future-law/repeating intents, complete history/grouping/clock, source/copies/output/legal/language/fulfillment remain owned.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="260">
+      <x:c r="A260" t="inlineStr">
+        <x:is>
+          <x:t>NY-FUTURE-APPLICATIONS-20261013</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B260" t="inlineStr">
+        <x:is>
+          <x:t>P02 / P03-09 / P04 / P09</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C260" t="inlineStr">
+        <x:is>
+          <x:t>NY</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D260" t="inlineStr">
+        <x:is>
+          <x:t>Intended future applications and explicit case/court associations</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E260" t="inlineStr">
+        <x:is>
+          <x:t>Intent does not establish eligibility, filing, source approval or output readiness</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F260" t="inlineStr">
+        <x:is>
+          <x:t>Exact historical successor, ENES ordinary-owner save/recovery and prior-order preservation</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G260" t="inlineStr">
+        <x:is>
+          <x:t>BOTH</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H260" t="inlineStr">
+        <x:is>
+          <x:t>PR268 after1842db25e</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I260" t="inlineStr">
+        <x:is>
+          <x:t>IN PROGRESS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J260" t="inlineStr">
+        <x:is>
+          <x:t>Bounded engineering checks PASS; future laws/repeated identities retained; stale and wrong-owner writes denied.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K260" t="inlineStr">
+        <x:is>
+          <x:t>ny-residual-20261012/FUTURE-RESTART-CHECKPOINT-v1.json</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L260" t="inlineStr">
+        <x:is>
+          <x:t>Codex engineering; preserved independent pure probe; qualified/final independent acceptance pending</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M260" t="inlineStr">
+        <x:is>
+          <x:t>GA-17 / GA-19 / GA-43 / GA-49</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N260" t="inlineStr">
+        <x:is>
+          <x:t>Full history/grouping/clock, authentic source/current widgets, copies/output/delivery and qualified legal/language/device review remain open.</x:t>
         </x:is>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Clarify Georgia First Offender next steps by case status
</commit_message>
<xml_diff>
--- a/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
+++ b/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
@@ -546,7 +546,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N260" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N261" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Case ID"/>
     <x:tableColumn id="2" name="Control ID"/>
@@ -26850,6 +26850,78 @@
       <x:c r="N260" t="inlineStr">
         <x:is>
           <x:t>Full history/grouping/clock, authentic source/current widgets, copies/output/delivery and qualified legal/language/device review remain open.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="261">
+      <x:c r="A261" t="inlineStr">
+        <x:is>
+          <x:t>GA-FIRST-OFFENDER-GUIDANCE-20261013</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B261" t="inlineStr">
+        <x:is>
+          <x:t>P02 / P04 / P09</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C261" t="inlineStr">
+        <x:is>
+          <x:t>GA</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D261" t="inlineStr">
+        <x:is>
+          <x:t>First Offender date/status-specific saved-result guidance</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E261" t="inlineStr">
+        <x:is>
+          <x:t>Four source distinctions with existing review/payment/packet holds unchanged</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F261" t="inlineStr">
+        <x:is>
+          <x:t>Public handler, genuine historical saved records, ordinary owner ENES correction across July1 cutoff</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G261" t="inlineStr">
+        <x:is>
+          <x:t>BOTH</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H261" t="inlineStr">
+        <x:is>
+          <x:t>PR268 afterdc50cd1ff7de</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I261" t="inlineStr">
+        <x:is>
+          <x:t>IN PROGRESS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J261" t="inlineStr">
+        <x:is>
+          <x:t>Engineering PASS: 5724 affected checks; owner EN147/ES151; exact restoration.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K261" t="inlineStr">
+        <x:is>
+          <x:t>ga-first-offender-guidance-20261013/GUIDANCE-CHECKPOINT-v1.json</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L261" t="inlineStr">
+        <x:is>
+          <x:t>Codex engineering; independent and qualified legal/language acceptance PENDING</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M261" t="inlineStr">
+        <x:is>
+          <x:t>GA-21 / GA-43</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N261" t="inlineStr">
+        <x:is>
+          <x:t>Full MS/GA/IL program/mixed/later-event predicates, contract/source review and remaining CX acceptance stay assigned. NY source/legal/document/delivery unchanged.</x:t>
         </x:is>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Translate shared Briefcase information-needed status
</commit_message>
<xml_diff>
--- a/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
+++ b/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
@@ -546,7 +546,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N261" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N262" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Case ID"/>
     <x:tableColumn id="2" name="Control ID"/>
@@ -26922,6 +26922,78 @@
       <x:c r="N261" t="inlineStr">
         <x:is>
           <x:t>Full MS/GA/IL program/mixed/later-event predicates, contract/source review and remaining CX acceptance stay assigned. NY source/legal/document/delivery unchanged.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="262">
+      <x:c r="A262" t="inlineStr">
+        <x:is>
+          <x:t>GA43-STATUS-GUIDANCE-20261013</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B262" t="inlineStr">
+        <x:is>
+          <x:t>P04 / P09</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C262" t="inlineStr">
+        <x:is>
+          <x:t>ALL (owner GA)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D262" t="inlineStr">
+        <x:is>
+          <x:t>Shared missing-information status heading and badge</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E262" t="inlineStr">
+        <x:is>
+          <x:t>Spanish titles and badges match the active locale; authority unchanged</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F262" t="inlineStr">
+        <x:is>
+          <x:t>Real humanMatterState producer for needs_review/needs_more_info; authenticated GA owner ENES</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G262" t="inlineStr">
+        <x:is>
+          <x:t>BOTH</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H262" t="inlineStr">
+        <x:is>
+          <x:t>PR268 afterd6badd7c5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I262" t="inlineStr">
+        <x:is>
+          <x:t>IN PROGRESS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J262" t="inlineStr">
+        <x:is>
+          <x:t>Two producer cases and155 GA regression checks PASS; owner EN39/ES39, exact restoration.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K262" t="inlineStr">
+        <x:is>
+          <x:t>ga43-status-guidance-20261013/STATUS-CHECKPOINT-v1.json</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L262" t="inlineStr">
+        <x:is>
+          <x:t>Codex engineering; independent language/device and full acceptance pending</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M262" t="inlineStr">
+        <x:is>
+          <x:t>GA-43</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N262" t="inlineStr">
+        <x:is>
+          <x:t>Remaining generated titles/subtitles/components, offered journeys and early-input hydration remain open; NY assignments unchanged.</x:t>
         </x:is>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Translate waiting and completed-facts Briefcase labels
</commit_message>
<xml_diff>
--- a/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
+++ b/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
@@ -546,7 +546,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N262" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N263" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Case ID"/>
     <x:tableColumn id="2" name="Control ID"/>
@@ -26994,6 +26994,78 @@
       <x:c r="N262" t="inlineStr">
         <x:is>
           <x:t>Remaining generated titles/subtitles/components, offered journeys and early-input hydration remain open; NY assignments unchanged.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="263">
+      <x:c r="A263" t="inlineStr">
+        <x:is>
+          <x:t>GA43-WAITING-FACTS-COPY-20261013</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B263" t="inlineStr">
+        <x:is>
+          <x:t>P04 / P09</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C263" t="inlineStr">
+        <x:is>
+          <x:t>ALL</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D263" t="inlineStr">
+        <x:is>
+          <x:t>Waiting/facts-complete shared status copy</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E263" t="inlineStr">
+        <x:is>
+          <x:t>Spanish display preserves the exact existing status meaning</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F263" t="inlineStr">
+        <x:is>
+          <x:t>Actual humanMatterState producer plus runtime resolver; no status/authority changes</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G263" t="inlineStr">
+        <x:is>
+          <x:t>BOTH</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H263" t="inlineStr">
+        <x:is>
+          <x:t>PR268 after76a5ba7dd</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I263" t="inlineStr">
+        <x:is>
+          <x:t>IN PROGRESS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J263" t="inlineStr">
+        <x:is>
+          <x:t>Two targeted producer cases fail before and pass after; lint/diff pass.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K263" t="inlineStr">
+        <x:is>
+          <x:t>ga43-waiting-facts-copy-20261013/COPY-CHECKPOINT-v1.json</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L263" t="inlineStr">
+        <x:is>
+          <x:t>Codex engineering; owner browser, independent language/device acceptance pending</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M263" t="inlineStr">
+        <x:is>
+          <x:t>GA-43</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N263" t="inlineStr">
+        <x:is>
+          <x:t>Remaining titles/subtitles/component labels, actual offered journeys and early-input timing remain assigned.</x:t>
         </x:is>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Integrate supplied NY and VA court sources as distinct review candidates
</commit_message>
<xml_diff>
--- a/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
+++ b/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
@@ -546,7 +546,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N263" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N265" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Case ID"/>
     <x:tableColumn id="2" name="Control ID"/>
@@ -642,7 +642,7 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="QASources" displayName="QASources" ref="A4:F17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="QASources" displayName="QASources" ref="A4:F21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="Source ID"/>
     <x:tableColumn id="2" name="Type"/>
@@ -27066,6 +27066,150 @@
       <x:c r="N263" t="inlineStr">
         <x:is>
           <x:t>Remaining titles/subtitles/component labels, actual offered journeys and early-input timing remain assigned.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="264">
+      <x:c r="A264" t="inlineStr">
+        <x:is>
+          <x:t>NY-CURRENT-SOURCE-INTAKE-20261013</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B264" t="inlineStr">
+        <x:is>
+          <x:t>P00 / P04</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C264" t="inlineStr">
+        <x:is>
+          <x:t>NY</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D264" t="inlineStr">
+        <x:is>
+          <x:t>August 2026 paper/fillable source custody and distinct draft maps</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E264" t="inlineStr">
+        <x:is>
+          <x:t>Keep current paper/fillable separate and preserve four historical pins</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F264" t="inlineStr">
+        <x:is>
+          <x:t>Owner ZIP verification, source widget census, paper anchors, protected preparation diagnostics</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G264" t="inlineStr">
+        <x:is>
+          <x:t>N/A source inspection</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H264" t="inlineStr">
+        <x:is>
+          <x:t>PR268 after ba8366343</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I264" t="inlineStr">
+        <x:is>
+          <x:t>IN PROGRESS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J264" t="inlineStr">
+        <x:is>
+          <x:t>Two NY originals verified; 84 widgets and 45 separate paper anchors; source guards10 plus NY971/927/2842 PASS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K264" t="inlineStr">
+        <x:is>
+          <x:t>court-source-handoff-20261013/ENGINEERING-CHECKPOINT-v1.json</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L264" t="inlineStr">
+        <x:is>
+          <x:t>Codex engineering; source custodian and qualified NY reviewer remain assigned</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M264" t="inlineStr">
+        <x:is>
+          <x:t>NY-SOURCE-CURRENT-01/02; GA-49</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N264" t="inlineStr">
+        <x:is>
+          <x:t>NY hosted copies HTTP403; historical four originals, qualified source/legal decisions, actual writes/rendering/visual and protected delivery remain outstanding.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="265">
+      <x:c r="A265" t="inlineStr">
+        <x:is>
+          <x:t>VA-SOURCE-MECHANISM-20261013</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B265" t="inlineStr">
+        <x:is>
+          <x:t>P00 / P04</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C265" t="inlineStr">
+        <x:is>
+          <x:t>VA</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D265" t="inlineStr">
+        <x:is>
+          <x:t>CC-1473 ordinary petition versus CC-1474A post-expungement access</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E265" t="inlineStr">
+        <x:is>
+          <x:t>Neither candidate may substitute for unresolved absolute-pardon procedure</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F265" t="inlineStr">
+        <x:is>
+          <x:t>Verify exact court downloads, existing CC1473 map and access-only draft</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G265" t="inlineStr">
+        <x:is>
+          <x:t>N/A source inspection</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H265" t="inlineStr">
+        <x:is>
+          <x:t>PR268 after ba8366343</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I265" t="inlineStr">
+        <x:is>
+          <x:t>IN PROGRESS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J265" t="inlineStr">
+        <x:is>
+          <x:t>Both supplied/hosted lengths and hashes match; CC1473 all42 prior widget mappings match; CC1474A25 widgets plus nonwidget court/signature blocks</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K265" t="inlineStr">
+        <x:is>
+          <x:t>court-source-handoff-20261013/ENGINEERING-CHECKPOINT-v1.json</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L265" t="inlineStr">
+        <x:is>
+          <x:t>Codex engineering; qualified VA source/legal review pending</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M265" t="inlineStr">
+        <x:is>
+          <x:t>GA-04 seven original assertion identities retained</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N265" t="inlineStr">
+        <x:is>
+          <x:t>No seven-fact closure or pardon instrument inferred; exact route binding, legal/source approvals, actual owner output and delivery remain outstanding.</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -30191,6 +30335,134 @@
         <x:v>Assurance checklist, not a claimed certification.</x:v>
       </x:c>
     </x:row>
+    <x:row r="18">
+      <x:c r="A18" t="inlineStr">
+        <x:is>
+          <x:t>COURT-20261013-01</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B18" t="inlineStr">
+        <x:is>
+          <x:t>Owner-supplied court source</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C18" t="inlineStr">
+        <x:is>
+          <x:t>https://www.vacourts.gov/static/forms/circuit/cc1473.pdf</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D18" t="inlineStr">
+        <x:is>
+          <x:t>petition_for_expungement_acquittal_dismissal</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E18" t="inlineStr">
+        <x:is>
+          <x:t>private/source-imports/court-source-handoff-20261013/source_files/cc1473.pdf | 120875 bytes | SHA256 6176c2f55bdb320682acecf0a79931bd5e496c4c93b5696645d4ef447fa67219</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F18" t="inlineStr">
+        <x:is>
+          <x:t>Supplied bytes verified; printed 07/26; hosted EXACT_MATCH. Qualified approval and production mapping NOT ACCEPTED. Separate originals preserved.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" t="inlineStr">
+        <x:is>
+          <x:t>COURT-20261013-02</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B19" t="inlineStr">
+        <x:is>
+          <x:t>Owner-supplied court source</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C19" t="inlineStr">
+        <x:is>
+          <x:t>https://www.vacourts.gov/static/forms/circuit/cc1474a.pdf</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D19" t="inlineStr">
+        <x:is>
+          <x:t>petition_to_access_already_expunged_record</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E19" t="inlineStr">
+        <x:is>
+          <x:t>private/source-imports/court-source-handoff-20261013/source_files/cc1474a.pdf | 101513 bytes | SHA256 7b8780ad50c029ec4d9a7db97ce7fe36f6a1fb05062bc37fd639348ac91c148d</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F19" t="inlineStr">
+        <x:is>
+          <x:t>Supplied bytes verified; printed 07/26; hosted EXACT_MATCH. Qualified approval and production mapping NOT ACCEPTED. Separate originals preserved.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" t="inlineStr">
+        <x:is>
+          <x:t>COURT-20261013-03</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B20" t="inlineStr">
+        <x:is>
+          <x:t>Owner-supplied court source</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C20" t="inlineStr">
+        <x:is>
+          <x:t>https://webfiles.nycourts.gov/public/2026-08/cpl160.59sealingapplication.pdf</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D20" t="inlineStr">
+        <x:is>
+          <x:t>current_paper_sealing_application</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E20" t="inlineStr">
+        <x:is>
+          <x:t>private/source-imports/court-source-handoff-20261013/source_files/cpl160.59sealingapplication.pdf | 283880 bytes | SHA256 4285ecff7baeed3acac3124cb16cf20b209259af1833e4a48967e6c1a61cec33</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F20" t="inlineStr">
+        <x:is>
+          <x:t>Supplied bytes verified; printed 08/2026; hosted UNAVAILABLE. Qualified approval and production mapping NOT ACCEPTED. Separate originals preserved.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" t="inlineStr">
+        <x:is>
+          <x:t>COURT-20261013-04</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B21" t="inlineStr">
+        <x:is>
+          <x:t>Owner-supplied court source</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C21" t="inlineStr">
+        <x:is>
+          <x:t>https://webfiles.nycourts.gov/public/2026-08/cpl160.59sealingapplication-fillable.pdf</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D21" t="inlineStr">
+        <x:is>
+          <x:t>current_fillable_sealing_application</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E21" t="inlineStr">
+        <x:is>
+          <x:t>private/source-imports/court-source-handoff-20261013/source_files/cpl160.59sealingapplication-fillable.pdf | 10689138 bytes | SHA256 633f06e1481d9c1a4b3ec987770eff577ac1147afeb3de0661b15c3ce659bccf</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F21" t="inlineStr">
+        <x:is>
+          <x:t>Supplied bytes verified; printed 08/2026; hosted UNAVAILABLE. Qualified approval and production mapping NOT ACCEPTED. Separate originals preserved.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:F1"/>

</xml_diff>

<commit_message>
Apply adopted GA-02 offense-class correction to pardon requests
</commit_message>
<xml_diff>
--- a/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
+++ b/qa/grade-a/ExpungementAI_Final_QA_Checklist.xlsx
@@ -546,7 +546,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N265" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QACases" displayName="QACases" ref="A4:N266" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Case ID"/>
     <x:tableColumn id="2" name="Control ID"/>
@@ -27210,6 +27210,78 @@
       <x:c r="N265" t="inlineStr">
         <x:is>
           <x:t>No seven-fact closure or pardon instrument inferred; exact route binding, legal/source approvals, actual owner output and delivery remain outstanding.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="266">
+      <x:c r="A266" t="inlineStr">
+        <x:is>
+          <x:t>GA02-ADOPTED-PARDON-PREDICATE-20261013</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B266" t="inlineStr">
+        <x:is>
+          <x:t>P03 / P04 / P09</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C266" t="inlineStr">
+        <x:is>
+          <x:t>GA</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D266" t="inlineStr">
+        <x:is>
+          <x:t>Adopted GA-02: offense classification cannot impose felony-only pardon eligibility</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E266" t="inlineStr">
+        <x:is>
+          <x:t>Explicit pardoned misdemeanor and felony select existing route; unknown class still clarified; no commercial permission</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F266" t="inlineStr">
+        <x:is>
+          <x:t>4226 affected checks,23 independent baseline/current checks; authenticated EN59/ES59 existing exact-source receipts revalidated</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G266" t="inlineStr">
+        <x:is>
+          <x:t>EN/ES isolated owner journeys; no hosted or language approval</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H266" t="inlineStr">
+        <x:is>
+          <x:t>PR268 verified candidate at f5449fcae</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I266" t="inlineStr">
+        <x:is>
+          <x:t>IN PROGRESS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J266" t="inlineStr">
+        <x:is>
+          <x:t>Baseline misdemeanor refusal reproduced; corrected predicate and request labels; raw answers and remaining gates preserved</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K266" t="inlineStr">
+        <x:is>
+          <x:t>counsel-adoption-20261013/GA02-INDEPENDENT-TECHNICAL-REVIEW-v1.json</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L266" t="inlineStr">
+        <x:is>
+          <x:t>Codex implementation; independent technical review; remaining product/document/language acceptance assigned</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M266" t="inlineStr">
+        <x:is>
+          <x:t>Legal decision GA-02; finding GA-42 / GA-43 (not original finding GA-02)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N266" t="inlineStr">
+        <x:is>
+          <x:t>Owner-relayed counsel adoption hash4ffc56d4 supersedes prior hash. Board-specific question, complete conditions/exceptions, participant route copy, document/language/hosted acceptance remain open.</x:t>
         </x:is>
       </x:c>
     </x:row>

</xml_diff>